<commit_message>
Correzioni da V07: modello nota spese e decadenza CPB in D01
- 04-roadmap/modelli/Nota-spese-trasferte.xlsx: soglia esente del
  forfettario calcolata per giorno; controllo sul comune della sede esteso a
  «Villafranca» e alle frazioni; regolamento trasferte approvato dai soci.
- 01-diagnosi/D01-diagnosi.md § 5.5: reati rilevanti anche nei tre periodi
  precedenti l'adesione; violazioni del sostituto non causa di decadenza.
- .gitignore: esclusa anche la verifica riservata V07.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/04-roadmap/modelli/Nota-spese-trasferte.xlsx
+++ b/04-roadmap/modelli/Nota-spese-trasferte.xlsx
@@ -726,12 +726,12 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Frazioni del comune della sede (separate da virgola)</t>
+          <t>Altri nomi e frazioni del comune della sede (separati da virgola)</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Alpo,Caluri,Dossobuono,Pizzoletta,Quaderni,Rizza,Rosegaferro</t>
+          <t>Villafranca,Alpo,Caluri,Dossobuono,Pizzoletta,Quaderni,Rizza,Rosegaferro</t>
         </is>
       </c>
     </row>
@@ -1738,7 +1738,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Alternativa al foglio «Nota spese»: usare solo se il regolamento trasferte prevede l'indennità forfettaria.</t>
+          <t>Alternativa al foglio «Nota spese»: solo per rimborsare trasferte reali, e solo se il regolamento trasferte approvato dai soci prevede l'indennità forfettaria. Non è un'integrazione del compenso.</t>
         </is>
       </c>
     </row>
@@ -1834,7 +1834,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Frazioni del comune della sede</t>
+          <t>Altri nomi e frazioni del comune della sede</t>
         </is>
       </c>
       <c r="C12" s="22">
@@ -1993,7 +1993,7 @@
         <v/>
       </c>
       <c r="O15" s="10">
-        <f>IF(A15="","",MIN(N15,IF(AND(N(K15)&gt;0,N(L15)&gt;0),$C$11,IF(OR(N(K15)&gt;0,N(L15)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A15="","",MIN(N15,IF(AND(SUMIF($A$15:$A$39,A15,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A15,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A15,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A15,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P15" s="10">
@@ -2034,7 +2034,7 @@
         <v/>
       </c>
       <c r="O16" s="14">
-        <f>IF(A16="","",MIN(N16,IF(AND(N(K16)&gt;0,N(L16)&gt;0),$C$11,IF(OR(N(K16)&gt;0,N(L16)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A16="","",MIN(N16,IF(AND(SUMIF($A$15:$A$39,A16,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A16,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A16,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A16,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P16" s="14">
@@ -2073,7 +2073,7 @@
         <v/>
       </c>
       <c r="O17" s="14">
-        <f>IF(A17="","",MIN(N17,IF(AND(N(K17)&gt;0,N(L17)&gt;0),$C$11,IF(OR(N(K17)&gt;0,N(L17)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A17="","",MIN(N17,IF(AND(SUMIF($A$15:$A$39,A17,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A17,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A17,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A17,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P17" s="14">
@@ -2112,7 +2112,7 @@
         <v/>
       </c>
       <c r="O18" s="14">
-        <f>IF(A18="","",MIN(N18,IF(AND(N(K18)&gt;0,N(L18)&gt;0),$C$11,IF(OR(N(K18)&gt;0,N(L18)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A18="","",MIN(N18,IF(AND(SUMIF($A$15:$A$39,A18,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A18,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A18,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A18,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P18" s="14">
@@ -2151,7 +2151,7 @@
         <v/>
       </c>
       <c r="O19" s="14">
-        <f>IF(A19="","",MIN(N19,IF(AND(N(K19)&gt;0,N(L19)&gt;0),$C$11,IF(OR(N(K19)&gt;0,N(L19)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A19="","",MIN(N19,IF(AND(SUMIF($A$15:$A$39,A19,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A19,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A19,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A19,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P19" s="14">
@@ -2190,7 +2190,7 @@
         <v/>
       </c>
       <c r="O20" s="14">
-        <f>IF(A20="","",MIN(N20,IF(AND(N(K20)&gt;0,N(L20)&gt;0),$C$11,IF(OR(N(K20)&gt;0,N(L20)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A20="","",MIN(N20,IF(AND(SUMIF($A$15:$A$39,A20,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A20,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A20,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A20,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P20" s="14">
@@ -2229,7 +2229,7 @@
         <v/>
       </c>
       <c r="O21" s="14">
-        <f>IF(A21="","",MIN(N21,IF(AND(N(K21)&gt;0,N(L21)&gt;0),$C$11,IF(OR(N(K21)&gt;0,N(L21)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A21="","",MIN(N21,IF(AND(SUMIF($A$15:$A$39,A21,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A21,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A21,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A21,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P21" s="14">
@@ -2268,7 +2268,7 @@
         <v/>
       </c>
       <c r="O22" s="14">
-        <f>IF(A22="","",MIN(N22,IF(AND(N(K22)&gt;0,N(L22)&gt;0),$C$11,IF(OR(N(K22)&gt;0,N(L22)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A22="","",MIN(N22,IF(AND(SUMIF($A$15:$A$39,A22,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A22,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A22,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A22,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P22" s="14">
@@ -2307,7 +2307,7 @@
         <v/>
       </c>
       <c r="O23" s="14">
-        <f>IF(A23="","",MIN(N23,IF(AND(N(K23)&gt;0,N(L23)&gt;0),$C$11,IF(OR(N(K23)&gt;0,N(L23)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A23="","",MIN(N23,IF(AND(SUMIF($A$15:$A$39,A23,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A23,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A23,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A23,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P23" s="14">
@@ -2346,7 +2346,7 @@
         <v/>
       </c>
       <c r="O24" s="14">
-        <f>IF(A24="","",MIN(N24,IF(AND(N(K24)&gt;0,N(L24)&gt;0),$C$11,IF(OR(N(K24)&gt;0,N(L24)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A24="","",MIN(N24,IF(AND(SUMIF($A$15:$A$39,A24,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A24,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A24,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A24,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P24" s="14">
@@ -2385,7 +2385,7 @@
         <v/>
       </c>
       <c r="O25" s="14">
-        <f>IF(A25="","",MIN(N25,IF(AND(N(K25)&gt;0,N(L25)&gt;0),$C$11,IF(OR(N(K25)&gt;0,N(L25)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A25="","",MIN(N25,IF(AND(SUMIF($A$15:$A$39,A25,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A25,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A25,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A25,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P25" s="14">
@@ -2424,7 +2424,7 @@
         <v/>
       </c>
       <c r="O26" s="14">
-        <f>IF(A26="","",MIN(N26,IF(AND(N(K26)&gt;0,N(L26)&gt;0),$C$11,IF(OR(N(K26)&gt;0,N(L26)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A26="","",MIN(N26,IF(AND(SUMIF($A$15:$A$39,A26,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A26,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A26,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A26,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P26" s="14">
@@ -2463,7 +2463,7 @@
         <v/>
       </c>
       <c r="O27" s="14">
-        <f>IF(A27="","",MIN(N27,IF(AND(N(K27)&gt;0,N(L27)&gt;0),$C$11,IF(OR(N(K27)&gt;0,N(L27)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A27="","",MIN(N27,IF(AND(SUMIF($A$15:$A$39,A27,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A27,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A27,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A27,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P27" s="14">
@@ -2502,7 +2502,7 @@
         <v/>
       </c>
       <c r="O28" s="14">
-        <f>IF(A28="","",MIN(N28,IF(AND(N(K28)&gt;0,N(L28)&gt;0),$C$11,IF(OR(N(K28)&gt;0,N(L28)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A28="","",MIN(N28,IF(AND(SUMIF($A$15:$A$39,A28,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A28,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A28,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A28,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P28" s="14">
@@ -2541,7 +2541,7 @@
         <v/>
       </c>
       <c r="O29" s="14">
-        <f>IF(A29="","",MIN(N29,IF(AND(N(K29)&gt;0,N(L29)&gt;0),$C$11,IF(OR(N(K29)&gt;0,N(L29)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A29="","",MIN(N29,IF(AND(SUMIF($A$15:$A$39,A29,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A29,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A29,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A29,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P29" s="14">
@@ -2580,7 +2580,7 @@
         <v/>
       </c>
       <c r="O30" s="14">
-        <f>IF(A30="","",MIN(N30,IF(AND(N(K30)&gt;0,N(L30)&gt;0),$C$11,IF(OR(N(K30)&gt;0,N(L30)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A30="","",MIN(N30,IF(AND(SUMIF($A$15:$A$39,A30,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A30,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A30,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A30,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P30" s="14">
@@ -2619,7 +2619,7 @@
         <v/>
       </c>
       <c r="O31" s="14">
-        <f>IF(A31="","",MIN(N31,IF(AND(N(K31)&gt;0,N(L31)&gt;0),$C$11,IF(OR(N(K31)&gt;0,N(L31)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A31="","",MIN(N31,IF(AND(SUMIF($A$15:$A$39,A31,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A31,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A31,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A31,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P31" s="14">
@@ -2658,7 +2658,7 @@
         <v/>
       </c>
       <c r="O32" s="14">
-        <f>IF(A32="","",MIN(N32,IF(AND(N(K32)&gt;0,N(L32)&gt;0),$C$11,IF(OR(N(K32)&gt;0,N(L32)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A32="","",MIN(N32,IF(AND(SUMIF($A$15:$A$39,A32,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A32,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A32,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A32,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P32" s="14">
@@ -2697,7 +2697,7 @@
         <v/>
       </c>
       <c r="O33" s="14">
-        <f>IF(A33="","",MIN(N33,IF(AND(N(K33)&gt;0,N(L33)&gt;0),$C$11,IF(OR(N(K33)&gt;0,N(L33)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A33="","",MIN(N33,IF(AND(SUMIF($A$15:$A$39,A33,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A33,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A33,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A33,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P33" s="14">
@@ -2736,7 +2736,7 @@
         <v/>
       </c>
       <c r="O34" s="14">
-        <f>IF(A34="","",MIN(N34,IF(AND(N(K34)&gt;0,N(L34)&gt;0),$C$11,IF(OR(N(K34)&gt;0,N(L34)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A34="","",MIN(N34,IF(AND(SUMIF($A$15:$A$39,A34,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A34,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A34,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A34,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P34" s="14">
@@ -2775,7 +2775,7 @@
         <v/>
       </c>
       <c r="O35" s="14">
-        <f>IF(A35="","",MIN(N35,IF(AND(N(K35)&gt;0,N(L35)&gt;0),$C$11,IF(OR(N(K35)&gt;0,N(L35)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A35="","",MIN(N35,IF(AND(SUMIF($A$15:$A$39,A35,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A35,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A35,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A35,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P35" s="14">
@@ -2814,7 +2814,7 @@
         <v/>
       </c>
       <c r="O36" s="14">
-        <f>IF(A36="","",MIN(N36,IF(AND(N(K36)&gt;0,N(L36)&gt;0),$C$11,IF(OR(N(K36)&gt;0,N(L36)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A36="","",MIN(N36,IF(AND(SUMIF($A$15:$A$39,A36,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A36,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A36,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A36,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P36" s="14">
@@ -2853,7 +2853,7 @@
         <v/>
       </c>
       <c r="O37" s="14">
-        <f>IF(A37="","",MIN(N37,IF(AND(N(K37)&gt;0,N(L37)&gt;0),$C$11,IF(OR(N(K37)&gt;0,N(L37)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A37="","",MIN(N37,IF(AND(SUMIF($A$15:$A$39,A37,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A37,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A37,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A37,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P37" s="14">
@@ -2892,7 +2892,7 @@
         <v/>
       </c>
       <c r="O38" s="14">
-        <f>IF(A38="","",MIN(N38,IF(AND(N(K38)&gt;0,N(L38)&gt;0),$C$11,IF(OR(N(K38)&gt;0,N(L38)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A38="","",MIN(N38,IF(AND(SUMIF($A$15:$A$39,A38,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A38,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A38,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A38,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P38" s="14">
@@ -2931,7 +2931,7 @@
         <v/>
       </c>
       <c r="O39" s="14">
-        <f>IF(A39="","",MIN(N39,IF(AND(N(K39)&gt;0,N(L39)&gt;0),$C$11,IF(OR(N(K39)&gt;0,N(L39)&gt;0),$C$10,$C$9))))</f>
+        <f>IF(A39="","",MIN(N39,IF(AND(SUMIF($A$15:$A$39,A39,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A39,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A39,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A39,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
       <c r="P39" s="14">
@@ -3266,7 +3266,7 @@
     <row r="25">
       <c r="A25" s="29" t="inlineStr">
         <is>
-          <t>Si usa uno solo dei due fogli, secondo quanto sceglie il regolamento trasferte deliberato dal CdA. Non si mescolano nello stesso mese.</t>
+          <t>Si usa uno solo dei due fogli, secondo quanto prevede il regolamento trasferte approvato dai soci. Non si mescolano nello stesso mese. L'indennità rimborsa trasferte reali: non serve a integrare il compenso.</t>
         </is>
       </c>
     </row>
@@ -3325,7 +3325,7 @@
     <row r="34">
       <c r="A34" s="29" t="inlineStr">
         <is>
-          <t>Presupposti da deliberare una volta dal CdA: sede di lavoro dell'amministratore a Villafranca di Verona; regolamento trasferte; approvazione delle note da parte di un altro amministratore.</t>
+          <t>Presupposti da approvare una volta dai soci (art. 24 dello statuto, trattamento degli amministratori): sede di lavoro dell'amministratore a Villafranca di Verona; regolamento trasferte; approvazione di ogni nota da parte di un altro amministratore.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Nota spese: riga di esempio esclusa dai totali, fogli protetti (V10 E-1, E-2)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/04-roadmap/modelli/Nota-spese-trasferte.xlsx
+++ b/04-roadmap/modelli/Nota-spese-trasferte.xlsx
@@ -155,20 +155,36 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="4" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
     <xf numFmtId="168" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="4" fillId="4" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
     <xf numFmtId="168" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="4" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -619,6 +635,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -735,6 +752,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
@@ -886,7 +904,7 @@
         <v/>
       </c>
       <c r="Q16" s="12">
-        <f>IF(A16="","",IF(OR(F16="",C16=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F16))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F16))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K16:M16)&gt;0,UPPER(N16)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O16&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A16="","",IF(ISNUMBER(SEARCH("ESEMPIO",B16)),"ESEMPIO: cancellare la riga",IF(OR(F16="",C16=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F16))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F16))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K16:M16)&gt;0,UPPER(N16)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O16&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -914,7 +932,7 @@
         <v/>
       </c>
       <c r="Q17" s="16">
-        <f>IF(A17="","",IF(OR(F17="",C17=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F17))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F17))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K17:M17)&gt;0,UPPER(N17)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O17&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A17="","",IF(ISNUMBER(SEARCH("ESEMPIO",B17)),"ESEMPIO: cancellare la riga",IF(OR(F17="",C17=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F17))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F17))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K17:M17)&gt;0,UPPER(N17)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O17&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -942,7 +960,7 @@
         <v/>
       </c>
       <c r="Q18" s="16">
-        <f>IF(A18="","",IF(OR(F18="",C18=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F18))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F18))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K18:M18)&gt;0,UPPER(N18)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O18&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A18="","",IF(ISNUMBER(SEARCH("ESEMPIO",B18)),"ESEMPIO: cancellare la riga",IF(OR(F18="",C18=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F18))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F18))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K18:M18)&gt;0,UPPER(N18)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O18&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -970,7 +988,7 @@
         <v/>
       </c>
       <c r="Q19" s="16">
-        <f>IF(A19="","",IF(OR(F19="",C19=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F19))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F19))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K19:M19)&gt;0,UPPER(N19)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O19&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A19="","",IF(ISNUMBER(SEARCH("ESEMPIO",B19)),"ESEMPIO: cancellare la riga",IF(OR(F19="",C19=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F19))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F19))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K19:M19)&gt;0,UPPER(N19)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O19&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -998,7 +1016,7 @@
         <v/>
       </c>
       <c r="Q20" s="16">
-        <f>IF(A20="","",IF(OR(F20="",C20=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F20))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F20))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K20:M20)&gt;0,UPPER(N20)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O20&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A20="","",IF(ISNUMBER(SEARCH("ESEMPIO",B20)),"ESEMPIO: cancellare la riga",IF(OR(F20="",C20=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F20))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F20))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K20:M20)&gt;0,UPPER(N20)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O20&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1026,7 +1044,7 @@
         <v/>
       </c>
       <c r="Q21" s="16">
-        <f>IF(A21="","",IF(OR(F21="",C21=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F21))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F21))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K21:M21)&gt;0,UPPER(N21)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O21&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A21="","",IF(ISNUMBER(SEARCH("ESEMPIO",B21)),"ESEMPIO: cancellare la riga",IF(OR(F21="",C21=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F21))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F21))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K21:M21)&gt;0,UPPER(N21)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O21&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1054,7 +1072,7 @@
         <v/>
       </c>
       <c r="Q22" s="16">
-        <f>IF(A22="","",IF(OR(F22="",C22=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F22))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F22))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K22:M22)&gt;0,UPPER(N22)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O22&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A22="","",IF(ISNUMBER(SEARCH("ESEMPIO",B22)),"ESEMPIO: cancellare la riga",IF(OR(F22="",C22=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F22))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F22))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K22:M22)&gt;0,UPPER(N22)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O22&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1082,7 +1100,7 @@
         <v/>
       </c>
       <c r="Q23" s="16">
-        <f>IF(A23="","",IF(OR(F23="",C23=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F23))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F23))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K23:M23)&gt;0,UPPER(N23)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O23&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A23="","",IF(ISNUMBER(SEARCH("ESEMPIO",B23)),"ESEMPIO: cancellare la riga",IF(OR(F23="",C23=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F23))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F23))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K23:M23)&gt;0,UPPER(N23)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O23&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1110,7 +1128,7 @@
         <v/>
       </c>
       <c r="Q24" s="16">
-        <f>IF(A24="","",IF(OR(F24="",C24=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F24))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F24))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K24:M24)&gt;0,UPPER(N24)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O24&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A24="","",IF(ISNUMBER(SEARCH("ESEMPIO",B24)),"ESEMPIO: cancellare la riga",IF(OR(F24="",C24=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F24))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F24))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K24:M24)&gt;0,UPPER(N24)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O24&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1138,7 +1156,7 @@
         <v/>
       </c>
       <c r="Q25" s="16">
-        <f>IF(A25="","",IF(OR(F25="",C25=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F25))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F25))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K25:M25)&gt;0,UPPER(N25)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O25&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A25="","",IF(ISNUMBER(SEARCH("ESEMPIO",B25)),"ESEMPIO: cancellare la riga",IF(OR(F25="",C25=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F25))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F25))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K25:M25)&gt;0,UPPER(N25)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O25&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1166,7 +1184,7 @@
         <v/>
       </c>
       <c r="Q26" s="16">
-        <f>IF(A26="","",IF(OR(F26="",C26=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F26))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F26))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K26:M26)&gt;0,UPPER(N26)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O26&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A26="","",IF(ISNUMBER(SEARCH("ESEMPIO",B26)),"ESEMPIO: cancellare la riga",IF(OR(F26="",C26=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F26))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F26))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K26:M26)&gt;0,UPPER(N26)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O26&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1194,7 +1212,7 @@
         <v/>
       </c>
       <c r="Q27" s="16">
-        <f>IF(A27="","",IF(OR(F27="",C27=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F27))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F27))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K27:M27)&gt;0,UPPER(N27)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O27&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A27="","",IF(ISNUMBER(SEARCH("ESEMPIO",B27)),"ESEMPIO: cancellare la riga",IF(OR(F27="",C27=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F27))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F27))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K27:M27)&gt;0,UPPER(N27)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O27&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1222,7 +1240,7 @@
         <v/>
       </c>
       <c r="Q28" s="16">
-        <f>IF(A28="","",IF(OR(F28="",C28=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F28))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F28))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K28:M28)&gt;0,UPPER(N28)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O28&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A28="","",IF(ISNUMBER(SEARCH("ESEMPIO",B28)),"ESEMPIO: cancellare la riga",IF(OR(F28="",C28=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F28))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F28))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K28:M28)&gt;0,UPPER(N28)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O28&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1250,7 +1268,7 @@
         <v/>
       </c>
       <c r="Q29" s="16">
-        <f>IF(A29="","",IF(OR(F29="",C29=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F29))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F29))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K29:M29)&gt;0,UPPER(N29)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O29&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A29="","",IF(ISNUMBER(SEARCH("ESEMPIO",B29)),"ESEMPIO: cancellare la riga",IF(OR(F29="",C29=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F29))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F29))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K29:M29)&gt;0,UPPER(N29)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O29&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1278,7 +1296,7 @@
         <v/>
       </c>
       <c r="Q30" s="16">
-        <f>IF(A30="","",IF(OR(F30="",C30=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F30))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F30))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K30:M30)&gt;0,UPPER(N30)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O30&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A30="","",IF(ISNUMBER(SEARCH("ESEMPIO",B30)),"ESEMPIO: cancellare la riga",IF(OR(F30="",C30=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F30))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F30))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K30:M30)&gt;0,UPPER(N30)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O30&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1306,7 +1324,7 @@
         <v/>
       </c>
       <c r="Q31" s="16">
-        <f>IF(A31="","",IF(OR(F31="",C31=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F31))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F31))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K31:M31)&gt;0,UPPER(N31)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O31&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A31="","",IF(ISNUMBER(SEARCH("ESEMPIO",B31)),"ESEMPIO: cancellare la riga",IF(OR(F31="",C31=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F31))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F31))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K31:M31)&gt;0,UPPER(N31)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O31&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1334,7 +1352,7 @@
         <v/>
       </c>
       <c r="Q32" s="16">
-        <f>IF(A32="","",IF(OR(F32="",C32=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F32))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F32))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K32:M32)&gt;0,UPPER(N32)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O32&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A32="","",IF(ISNUMBER(SEARCH("ESEMPIO",B32)),"ESEMPIO: cancellare la riga",IF(OR(F32="",C32=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F32))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F32))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K32:M32)&gt;0,UPPER(N32)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O32&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1362,7 +1380,7 @@
         <v/>
       </c>
       <c r="Q33" s="16">
-        <f>IF(A33="","",IF(OR(F33="",C33=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F33))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F33))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K33:M33)&gt;0,UPPER(N33)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O33&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A33="","",IF(ISNUMBER(SEARCH("ESEMPIO",B33)),"ESEMPIO: cancellare la riga",IF(OR(F33="",C33=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F33))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F33))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K33:M33)&gt;0,UPPER(N33)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O33&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1390,7 +1408,7 @@
         <v/>
       </c>
       <c r="Q34" s="16">
-        <f>IF(A34="","",IF(OR(F34="",C34=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F34))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F34))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K34:M34)&gt;0,UPPER(N34)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O34&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A34="","",IF(ISNUMBER(SEARCH("ESEMPIO",B34)),"ESEMPIO: cancellare la riga",IF(OR(F34="",C34=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F34))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F34))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K34:M34)&gt;0,UPPER(N34)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O34&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1418,7 +1436,7 @@
         <v/>
       </c>
       <c r="Q35" s="16">
-        <f>IF(A35="","",IF(OR(F35="",C35=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F35))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F35))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K35:M35)&gt;0,UPPER(N35)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O35&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A35="","",IF(ISNUMBER(SEARCH("ESEMPIO",B35)),"ESEMPIO: cancellare la riga",IF(OR(F35="",C35=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F35))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F35))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K35:M35)&gt;0,UPPER(N35)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O35&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1446,7 +1464,7 @@
         <v/>
       </c>
       <c r="Q36" s="16">
-        <f>IF(A36="","",IF(OR(F36="",C36=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F36))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F36))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K36:M36)&gt;0,UPPER(N36)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O36&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A36="","",IF(ISNUMBER(SEARCH("ESEMPIO",B36)),"ESEMPIO: cancellare la riga",IF(OR(F36="",C36=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F36))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F36))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K36:M36)&gt;0,UPPER(N36)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O36&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1474,7 +1492,7 @@
         <v/>
       </c>
       <c r="Q37" s="16">
-        <f>IF(A37="","",IF(OR(F37="",C37=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F37))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F37))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K37:M37)&gt;0,UPPER(N37)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O37&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A37="","",IF(ISNUMBER(SEARCH("ESEMPIO",B37)),"ESEMPIO: cancellare la riga",IF(OR(F37="",C37=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F37))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F37))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K37:M37)&gt;0,UPPER(N37)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O37&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1502,7 +1520,7 @@
         <v/>
       </c>
       <c r="Q38" s="16">
-        <f>IF(A38="","",IF(OR(F38="",C38=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F38))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F38))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K38:M38)&gt;0,UPPER(N38)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O38&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A38="","",IF(ISNUMBER(SEARCH("ESEMPIO",B38)),"ESEMPIO: cancellare la riga",IF(OR(F38="",C38=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F38))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F38))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K38:M38)&gt;0,UPPER(N38)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O38&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1530,7 +1548,7 @@
         <v/>
       </c>
       <c r="Q39" s="16">
-        <f>IF(A39="","",IF(OR(F39="",C39=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F39))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F39))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K39:M39)&gt;0,UPPER(N39)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O39&lt;1,"MANCA allegato","OK")))))</f>
+        <f>IF(A39="","",IF(ISNUMBER(SEARCH("ESEMPIO",B39)),"ESEMPIO: cancellare la riga",IF(OR(F39="",C39=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F39))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F39))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K39:M39)&gt;0,UPPER(N39)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O39&lt;1,"MANCA allegato","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -1558,10 +1576,11 @@
         <v/>
       </c>
       <c r="Q40" s="16">
-        <f>IF(A40="","",IF(OR(F40="",C40=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F40))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F40))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K40:M40)&gt;0,UPPER(N40)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O40&lt;1,"MANCA allegato","OK")))))</f>
-        <v/>
-      </c>
-    </row>
+        <f>IF(A40="","",IF(ISNUMBER(SEARCH("ESEMPIO",B40)),"ESEMPIO: cancellare la riga",IF(OR(F40="",C40=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F40))=LOWER(TRIM($C$7)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F40))&amp;",",","&amp;LOWER(SUBSTITUTE($C$13," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(SUM(K40:M40)&gt;0,UPPER(N40)&lt;&gt;"S"),"NO: vitto/alloggio/taxi non tracciabile",IF(O40&lt;1,"MANCA allegato","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41"/>
     <row r="42">
       <c r="F42" s="3" t="inlineStr">
         <is>
@@ -1623,6 +1642,8 @@
         <v/>
       </c>
     </row>
+    <row r="45"/>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
@@ -1635,6 +1656,7 @@
       <c r="F47" s="21" t="n"/>
       <c r="G47" s="21" t="n"/>
     </row>
+    <row r="48"/>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
@@ -1647,6 +1669,7 @@
       <c r="F49" s="21" t="n"/>
       <c r="G49" s="21" t="n"/>
     </row>
+    <row r="50"/>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
@@ -1659,6 +1682,7 @@
       <c r="F51" s="21" t="n"/>
       <c r="G51" s="21" t="n"/>
     </row>
+    <row r="52"/>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
@@ -1672,6 +1696,7 @@
       <c r="G53" s="21" t="n"/>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
   <conditionalFormatting sqref="Q16:Q40">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>LEFT(Q16,2)="OK"</formula>
@@ -1742,6 +1767,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1842,6 +1868,7 @@
         <v/>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
@@ -2008,7 +2035,7 @@
         <v/>
       </c>
       <c r="S15" s="12">
-        <f>IF(A15="","",IF(OR(F15="",C15=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F15))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F15))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K15)+N(L15)&gt;0,UPPER(M15)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q15&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A15="","",IF(ISNUMBER(SEARCH("ESEMPIO",B15)),"ESEMPIO: cancellare la riga",IF(OR(F15="",C15=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F15))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F15))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K15)+N(L15)&gt;0,UPPER(M15)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q15&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2047,7 +2074,7 @@
         <v/>
       </c>
       <c r="S16" s="16">
-        <f>IF(A16="","",IF(OR(F16="",C16=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F16))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F16))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K16)+N(L16)&gt;0,UPPER(M16)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q16&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A16="","",IF(ISNUMBER(SEARCH("ESEMPIO",B16)),"ESEMPIO: cancellare la riga",IF(OR(F16="",C16=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F16))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F16))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K16)+N(L16)&gt;0,UPPER(M16)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q16&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2086,7 +2113,7 @@
         <v/>
       </c>
       <c r="S17" s="16">
-        <f>IF(A17="","",IF(OR(F17="",C17=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F17))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F17))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K17)+N(L17)&gt;0,UPPER(M17)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q17&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A17="","",IF(ISNUMBER(SEARCH("ESEMPIO",B17)),"ESEMPIO: cancellare la riga",IF(OR(F17="",C17=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F17))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F17))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K17)+N(L17)&gt;0,UPPER(M17)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q17&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2125,7 +2152,7 @@
         <v/>
       </c>
       <c r="S18" s="16">
-        <f>IF(A18="","",IF(OR(F18="",C18=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F18))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F18))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K18)+N(L18)&gt;0,UPPER(M18)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q18&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A18="","",IF(ISNUMBER(SEARCH("ESEMPIO",B18)),"ESEMPIO: cancellare la riga",IF(OR(F18="",C18=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F18))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F18))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K18)+N(L18)&gt;0,UPPER(M18)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q18&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2164,7 +2191,7 @@
         <v/>
       </c>
       <c r="S19" s="16">
-        <f>IF(A19="","",IF(OR(F19="",C19=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F19))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F19))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K19)+N(L19)&gt;0,UPPER(M19)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q19&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A19="","",IF(ISNUMBER(SEARCH("ESEMPIO",B19)),"ESEMPIO: cancellare la riga",IF(OR(F19="",C19=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F19))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F19))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K19)+N(L19)&gt;0,UPPER(M19)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q19&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2203,7 +2230,7 @@
         <v/>
       </c>
       <c r="S20" s="16">
-        <f>IF(A20="","",IF(OR(F20="",C20=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F20))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F20))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K20)+N(L20)&gt;0,UPPER(M20)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q20&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A20="","",IF(ISNUMBER(SEARCH("ESEMPIO",B20)),"ESEMPIO: cancellare la riga",IF(OR(F20="",C20=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F20))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F20))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K20)+N(L20)&gt;0,UPPER(M20)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q20&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2242,7 +2269,7 @@
         <v/>
       </c>
       <c r="S21" s="16">
-        <f>IF(A21="","",IF(OR(F21="",C21=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F21))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F21))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K21)+N(L21)&gt;0,UPPER(M21)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q21&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A21="","",IF(ISNUMBER(SEARCH("ESEMPIO",B21)),"ESEMPIO: cancellare la riga",IF(OR(F21="",C21=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F21))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F21))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K21)+N(L21)&gt;0,UPPER(M21)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q21&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2281,7 +2308,7 @@
         <v/>
       </c>
       <c r="S22" s="16">
-        <f>IF(A22="","",IF(OR(F22="",C22=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F22))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F22))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K22)+N(L22)&gt;0,UPPER(M22)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q22&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A22="","",IF(ISNUMBER(SEARCH("ESEMPIO",B22)),"ESEMPIO: cancellare la riga",IF(OR(F22="",C22=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F22))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F22))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K22)+N(L22)&gt;0,UPPER(M22)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q22&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2320,7 +2347,7 @@
         <v/>
       </c>
       <c r="S23" s="16">
-        <f>IF(A23="","",IF(OR(F23="",C23=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F23))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F23))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K23)+N(L23)&gt;0,UPPER(M23)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q23&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A23="","",IF(ISNUMBER(SEARCH("ESEMPIO",B23)),"ESEMPIO: cancellare la riga",IF(OR(F23="",C23=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F23))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F23))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K23)+N(L23)&gt;0,UPPER(M23)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q23&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2359,7 +2386,7 @@
         <v/>
       </c>
       <c r="S24" s="16">
-        <f>IF(A24="","",IF(OR(F24="",C24=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F24))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F24))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K24)+N(L24)&gt;0,UPPER(M24)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q24&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A24="","",IF(ISNUMBER(SEARCH("ESEMPIO",B24)),"ESEMPIO: cancellare la riga",IF(OR(F24="",C24=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F24))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F24))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K24)+N(L24)&gt;0,UPPER(M24)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q24&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2398,7 +2425,7 @@
         <v/>
       </c>
       <c r="S25" s="16">
-        <f>IF(A25="","",IF(OR(F25="",C25=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F25))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F25))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K25)+N(L25)&gt;0,UPPER(M25)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q25&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A25="","",IF(ISNUMBER(SEARCH("ESEMPIO",B25)),"ESEMPIO: cancellare la riga",IF(OR(F25="",C25=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F25))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F25))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K25)+N(L25)&gt;0,UPPER(M25)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q25&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2437,7 +2464,7 @@
         <v/>
       </c>
       <c r="S26" s="16">
-        <f>IF(A26="","",IF(OR(F26="",C26=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F26))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F26))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K26)+N(L26)&gt;0,UPPER(M26)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q26&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A26="","",IF(ISNUMBER(SEARCH("ESEMPIO",B26)),"ESEMPIO: cancellare la riga",IF(OR(F26="",C26=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F26))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F26))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K26)+N(L26)&gt;0,UPPER(M26)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q26&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2476,7 +2503,7 @@
         <v/>
       </c>
       <c r="S27" s="16">
-        <f>IF(A27="","",IF(OR(F27="",C27=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F27))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F27))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K27)+N(L27)&gt;0,UPPER(M27)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q27&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A27="","",IF(ISNUMBER(SEARCH("ESEMPIO",B27)),"ESEMPIO: cancellare la riga",IF(OR(F27="",C27=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F27))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F27))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K27)+N(L27)&gt;0,UPPER(M27)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q27&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2515,7 +2542,7 @@
         <v/>
       </c>
       <c r="S28" s="16">
-        <f>IF(A28="","",IF(OR(F28="",C28=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F28))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F28))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K28)+N(L28)&gt;0,UPPER(M28)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q28&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A28="","",IF(ISNUMBER(SEARCH("ESEMPIO",B28)),"ESEMPIO: cancellare la riga",IF(OR(F28="",C28=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F28))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F28))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K28)+N(L28)&gt;0,UPPER(M28)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q28&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2554,7 +2581,7 @@
         <v/>
       </c>
       <c r="S29" s="16">
-        <f>IF(A29="","",IF(OR(F29="",C29=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F29))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F29))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K29)+N(L29)&gt;0,UPPER(M29)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q29&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A29="","",IF(ISNUMBER(SEARCH("ESEMPIO",B29)),"ESEMPIO: cancellare la riga",IF(OR(F29="",C29=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F29))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F29))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K29)+N(L29)&gt;0,UPPER(M29)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q29&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2593,7 +2620,7 @@
         <v/>
       </c>
       <c r="S30" s="16">
-        <f>IF(A30="","",IF(OR(F30="",C30=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F30))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F30))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K30)+N(L30)&gt;0,UPPER(M30)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q30&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A30="","",IF(ISNUMBER(SEARCH("ESEMPIO",B30)),"ESEMPIO: cancellare la riga",IF(OR(F30="",C30=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F30))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F30))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K30)+N(L30)&gt;0,UPPER(M30)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q30&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2632,7 +2659,7 @@
         <v/>
       </c>
       <c r="S31" s="16">
-        <f>IF(A31="","",IF(OR(F31="",C31=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F31))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F31))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K31)+N(L31)&gt;0,UPPER(M31)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q31&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A31="","",IF(ISNUMBER(SEARCH("ESEMPIO",B31)),"ESEMPIO: cancellare la riga",IF(OR(F31="",C31=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F31))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F31))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K31)+N(L31)&gt;0,UPPER(M31)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q31&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2671,7 +2698,7 @@
         <v/>
       </c>
       <c r="S32" s="16">
-        <f>IF(A32="","",IF(OR(F32="",C32=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F32))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F32))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K32)+N(L32)&gt;0,UPPER(M32)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q32&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A32="","",IF(ISNUMBER(SEARCH("ESEMPIO",B32)),"ESEMPIO: cancellare la riga",IF(OR(F32="",C32=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F32))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F32))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K32)+N(L32)&gt;0,UPPER(M32)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q32&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2710,7 +2737,7 @@
         <v/>
       </c>
       <c r="S33" s="16">
-        <f>IF(A33="","",IF(OR(F33="",C33=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F33))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F33))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K33)+N(L33)&gt;0,UPPER(M33)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q33&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A33="","",IF(ISNUMBER(SEARCH("ESEMPIO",B33)),"ESEMPIO: cancellare la riga",IF(OR(F33="",C33=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F33))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F33))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K33)+N(L33)&gt;0,UPPER(M33)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q33&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2749,7 +2776,7 @@
         <v/>
       </c>
       <c r="S34" s="16">
-        <f>IF(A34="","",IF(OR(F34="",C34=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F34))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F34))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K34)+N(L34)&gt;0,UPPER(M34)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q34&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A34="","",IF(ISNUMBER(SEARCH("ESEMPIO",B34)),"ESEMPIO: cancellare la riga",IF(OR(F34="",C34=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F34))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F34))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K34)+N(L34)&gt;0,UPPER(M34)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q34&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2788,7 +2815,7 @@
         <v/>
       </c>
       <c r="S35" s="16">
-        <f>IF(A35="","",IF(OR(F35="",C35=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F35))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F35))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K35)+N(L35)&gt;0,UPPER(M35)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q35&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A35="","",IF(ISNUMBER(SEARCH("ESEMPIO",B35)),"ESEMPIO: cancellare la riga",IF(OR(F35="",C35=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F35))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F35))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K35)+N(L35)&gt;0,UPPER(M35)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q35&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2827,7 +2854,7 @@
         <v/>
       </c>
       <c r="S36" s="16">
-        <f>IF(A36="","",IF(OR(F36="",C36=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F36))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F36))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K36)+N(L36)&gt;0,UPPER(M36)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q36&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A36="","",IF(ISNUMBER(SEARCH("ESEMPIO",B36)),"ESEMPIO: cancellare la riga",IF(OR(F36="",C36=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F36))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F36))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K36)+N(L36)&gt;0,UPPER(M36)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q36&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2866,7 +2893,7 @@
         <v/>
       </c>
       <c r="S37" s="16">
-        <f>IF(A37="","",IF(OR(F37="",C37=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F37))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F37))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K37)+N(L37)&gt;0,UPPER(M37)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q37&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A37="","",IF(ISNUMBER(SEARCH("ESEMPIO",B37)),"ESEMPIO: cancellare la riga",IF(OR(F37="",C37=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F37))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F37))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K37)+N(L37)&gt;0,UPPER(M37)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q37&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2905,7 +2932,7 @@
         <v/>
       </c>
       <c r="S38" s="16">
-        <f>IF(A38="","",IF(OR(F38="",C38=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F38))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F38))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K38)+N(L38)&gt;0,UPPER(M38)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q38&lt;1,"MANCA prova della trasferta","OK")))))</f>
+        <f>IF(A38="","",IF(ISNUMBER(SEARCH("ESEMPIO",B38)),"ESEMPIO: cancellare la riga",IF(OR(F38="",C38=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F38))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F38))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K38)+N(L38)&gt;0,UPPER(M38)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q38&lt;1,"MANCA prova della trasferta","OK"))))))</f>
         <v/>
       </c>
     </row>
@@ -2944,10 +2971,11 @@
         <v/>
       </c>
       <c r="S39" s="16">
-        <f>IF(A39="","",IF(OR(F39="",C39=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F39))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F39))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K39)+N(L39)&gt;0,UPPER(M39)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q39&lt;1,"MANCA prova della trasferta","OK")))))</f>
-        <v/>
-      </c>
-    </row>
+        <f>IF(A39="","",IF(ISNUMBER(SEARCH("ESEMPIO",B39)),"ESEMPIO: cancellare la riga",IF(OR(F39="",C39=""),"MANCA destinazione o commessa",IF(OR(LOWER(TRIM(F39))=LOWER(TRIM($C$6)),ISNUMBER(SEARCH(","&amp;LOWER(TRIM(F39))&amp;",",","&amp;LOWER(SUBSTITUTE($C$12," ",""))&amp;","))),"NO: trasferta nel comune della sede (o frazione)",IF(AND(N(K39)+N(L39)&gt;0,UPPER(M39)&lt;&gt;"S"),"NO: vitto/alloggio non tracciabile",IF(Q39&lt;1,"MANCA prova della trasferta","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40"/>
     <row r="41">
       <c r="F41" s="3" t="inlineStr">
         <is>
@@ -3028,6 +3056,8 @@
         <v/>
       </c>
     </row>
+    <row r="45"/>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
@@ -3040,6 +3070,7 @@
       <c r="F47" s="21" t="n"/>
       <c r="G47" s="21" t="n"/>
     </row>
+    <row r="48"/>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
@@ -3052,6 +3083,7 @@
       <c r="F49" s="21" t="n"/>
       <c r="G49" s="21" t="n"/>
     </row>
+    <row r="50"/>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
@@ -3064,6 +3096,7 @@
       <c r="F51" s="21" t="n"/>
       <c r="G51" s="21" t="n"/>
     </row>
+    <row r="52"/>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
@@ -3077,6 +3110,7 @@
       <c r="G53" s="21" t="n"/>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
   <conditionalFormatting sqref="S15:S39">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>LEFT(S15,2)="OK"</formula>
@@ -3337,6 +3371,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Guida alla compilazione della nota spese; istruzioni Excel più neutre
- 04-roadmap/modelli/Guida-compilazione-nota-spese.docx: guida pratica per
  il Presidente (quando la trasferta è rimborsabile, colonna per colonna,
  allegati, cosa non va in nota, controllo prima di firmare, fine mese).
  Recepisce la verifica indipendente; segnaposto in giallo da completare
  con le decisioni del 20/10.
- Nota-spese-trasferte.xlsx, foglio Istruzioni: righe 18, 20 e 22
  riformulate in modo neutro.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/04-roadmap/modelli/Nota-spese-trasferte.xlsx
+++ b/04-roadmap/modelli/Nota-spese-trasferte.xlsx
@@ -18,12 +18,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="mmmm yyyy"/>
-    <numFmt numFmtId="166" formatCode="0.0000"/>
-    <numFmt numFmtId="167" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="168" formatCode="#,##0.00;-#,##0.00;-"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="mmmm yyyy"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="167" formatCode="#,##0.00;-#,##0.00;-"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -150,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -158,51 +157,77 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="4" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="4" fillId="4" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="4" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="4" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="168" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="4" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="4" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="2" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -635,7 +660,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -666,7 +690,7 @@
           <t>Mese di riferimento</t>
         </is>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="30" t="n">
         <v>46082</v>
       </c>
     </row>
@@ -724,7 +748,7 @@
           <t>Tariffa ACI €/km del veicolo</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n">
+      <c r="C11" s="31" t="n">
         <v>0.45</v>
       </c>
     </row>
@@ -752,7 +776,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
@@ -841,7 +864,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="n">
+      <c r="A16" s="32" t="n">
         <v>46093</v>
       </c>
       <c r="B16" s="9" t="inlineStr">
@@ -872,23 +895,23 @@
       <c r="G16" s="9" t="n">
         <v>150</v>
       </c>
-      <c r="H16" s="10">
+      <c r="H16" s="33">
         <f>IF(G16="","",G16*$C$11)</f>
         <v/>
       </c>
-      <c r="I16" s="11" t="n">
+      <c r="I16" s="34" t="n">
         <v>10.4</v>
       </c>
-      <c r="J16" s="11" t="n">
+      <c r="J16" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="K16" s="11" t="n">
+      <c r="K16" s="34" t="n">
         <v>18</v>
       </c>
-      <c r="L16" s="11" t="n">
+      <c r="L16" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="M16" s="11" t="n">
+      <c r="M16" s="34" t="n">
         <v>0</v>
       </c>
       <c r="N16" s="9" t="inlineStr">
@@ -899,7 +922,7 @@
       <c r="O16" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="P16" s="10">
+      <c r="P16" s="33">
         <f>IF(A16="","",N(H16)+SUM(I16:M16))</f>
         <v/>
       </c>
@@ -909,25 +932,25 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="n"/>
+      <c r="A17" s="35" t="n"/>
       <c r="B17" s="4" t="n"/>
       <c r="C17" s="4" t="n"/>
       <c r="D17" s="4" t="n"/>
       <c r="E17" s="4" t="n"/>
       <c r="F17" s="4" t="n"/>
       <c r="G17" s="4" t="n"/>
-      <c r="H17" s="14">
+      <c r="H17" s="36">
         <f>IF(G17="","",G17*$C$11)</f>
         <v/>
       </c>
-      <c r="I17" s="15" t="n"/>
-      <c r="J17" s="15" t="n"/>
-      <c r="K17" s="15" t="n"/>
-      <c r="L17" s="15" t="n"/>
-      <c r="M17" s="15" t="n"/>
+      <c r="I17" s="37" t="n"/>
+      <c r="J17" s="37" t="n"/>
+      <c r="K17" s="37" t="n"/>
+      <c r="L17" s="37" t="n"/>
+      <c r="M17" s="37" t="n"/>
       <c r="N17" s="4" t="n"/>
       <c r="O17" s="4" t="n"/>
-      <c r="P17" s="14">
+      <c r="P17" s="36">
         <f>IF(A17="","",N(H17)+SUM(I17:M17))</f>
         <v/>
       </c>
@@ -937,25 +960,25 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="n"/>
+      <c r="A18" s="35" t="n"/>
       <c r="B18" s="4" t="n"/>
       <c r="C18" s="4" t="n"/>
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="4" t="n"/>
       <c r="F18" s="4" t="n"/>
       <c r="G18" s="4" t="n"/>
-      <c r="H18" s="14">
+      <c r="H18" s="36">
         <f>IF(G18="","",G18*$C$11)</f>
         <v/>
       </c>
-      <c r="I18" s="15" t="n"/>
-      <c r="J18" s="15" t="n"/>
-      <c r="K18" s="15" t="n"/>
-      <c r="L18" s="15" t="n"/>
-      <c r="M18" s="15" t="n"/>
+      <c r="I18" s="37" t="n"/>
+      <c r="J18" s="37" t="n"/>
+      <c r="K18" s="37" t="n"/>
+      <c r="L18" s="37" t="n"/>
+      <c r="M18" s="37" t="n"/>
       <c r="N18" s="4" t="n"/>
       <c r="O18" s="4" t="n"/>
-      <c r="P18" s="14">
+      <c r="P18" s="36">
         <f>IF(A18="","",N(H18)+SUM(I18:M18))</f>
         <v/>
       </c>
@@ -965,25 +988,25 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="n"/>
+      <c r="A19" s="35" t="n"/>
       <c r="B19" s="4" t="n"/>
       <c r="C19" s="4" t="n"/>
       <c r="D19" s="4" t="n"/>
       <c r="E19" s="4" t="n"/>
       <c r="F19" s="4" t="n"/>
       <c r="G19" s="4" t="n"/>
-      <c r="H19" s="14">
+      <c r="H19" s="36">
         <f>IF(G19="","",G19*$C$11)</f>
         <v/>
       </c>
-      <c r="I19" s="15" t="n"/>
-      <c r="J19" s="15" t="n"/>
-      <c r="K19" s="15" t="n"/>
-      <c r="L19" s="15" t="n"/>
-      <c r="M19" s="15" t="n"/>
+      <c r="I19" s="37" t="n"/>
+      <c r="J19" s="37" t="n"/>
+      <c r="K19" s="37" t="n"/>
+      <c r="L19" s="37" t="n"/>
+      <c r="M19" s="37" t="n"/>
       <c r="N19" s="4" t="n"/>
       <c r="O19" s="4" t="n"/>
-      <c r="P19" s="14">
+      <c r="P19" s="36">
         <f>IF(A19="","",N(H19)+SUM(I19:M19))</f>
         <v/>
       </c>
@@ -993,25 +1016,25 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="n"/>
+      <c r="A20" s="35" t="n"/>
       <c r="B20" s="4" t="n"/>
       <c r="C20" s="4" t="n"/>
       <c r="D20" s="4" t="n"/>
       <c r="E20" s="4" t="n"/>
       <c r="F20" s="4" t="n"/>
       <c r="G20" s="4" t="n"/>
-      <c r="H20" s="14">
+      <c r="H20" s="36">
         <f>IF(G20="","",G20*$C$11)</f>
         <v/>
       </c>
-      <c r="I20" s="15" t="n"/>
-      <c r="J20" s="15" t="n"/>
-      <c r="K20" s="15" t="n"/>
-      <c r="L20" s="15" t="n"/>
-      <c r="M20" s="15" t="n"/>
+      <c r="I20" s="37" t="n"/>
+      <c r="J20" s="37" t="n"/>
+      <c r="K20" s="37" t="n"/>
+      <c r="L20" s="37" t="n"/>
+      <c r="M20" s="37" t="n"/>
       <c r="N20" s="4" t="n"/>
       <c r="O20" s="4" t="n"/>
-      <c r="P20" s="14">
+      <c r="P20" s="36">
         <f>IF(A20="","",N(H20)+SUM(I20:M20))</f>
         <v/>
       </c>
@@ -1021,25 +1044,25 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="n"/>
+      <c r="A21" s="35" t="n"/>
       <c r="B21" s="4" t="n"/>
       <c r="C21" s="4" t="n"/>
       <c r="D21" s="4" t="n"/>
       <c r="E21" s="4" t="n"/>
       <c r="F21" s="4" t="n"/>
       <c r="G21" s="4" t="n"/>
-      <c r="H21" s="14">
+      <c r="H21" s="36">
         <f>IF(G21="","",G21*$C$11)</f>
         <v/>
       </c>
-      <c r="I21" s="15" t="n"/>
-      <c r="J21" s="15" t="n"/>
-      <c r="K21" s="15" t="n"/>
-      <c r="L21" s="15" t="n"/>
-      <c r="M21" s="15" t="n"/>
+      <c r="I21" s="37" t="n"/>
+      <c r="J21" s="37" t="n"/>
+      <c r="K21" s="37" t="n"/>
+      <c r="L21" s="37" t="n"/>
+      <c r="M21" s="37" t="n"/>
       <c r="N21" s="4" t="n"/>
       <c r="O21" s="4" t="n"/>
-      <c r="P21" s="14">
+      <c r="P21" s="36">
         <f>IF(A21="","",N(H21)+SUM(I21:M21))</f>
         <v/>
       </c>
@@ -1049,25 +1072,25 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="n"/>
+      <c r="A22" s="35" t="n"/>
       <c r="B22" s="4" t="n"/>
       <c r="C22" s="4" t="n"/>
       <c r="D22" s="4" t="n"/>
       <c r="E22" s="4" t="n"/>
       <c r="F22" s="4" t="n"/>
       <c r="G22" s="4" t="n"/>
-      <c r="H22" s="14">
+      <c r="H22" s="36">
         <f>IF(G22="","",G22*$C$11)</f>
         <v/>
       </c>
-      <c r="I22" s="15" t="n"/>
-      <c r="J22" s="15" t="n"/>
-      <c r="K22" s="15" t="n"/>
-      <c r="L22" s="15" t="n"/>
-      <c r="M22" s="15" t="n"/>
+      <c r="I22" s="37" t="n"/>
+      <c r="J22" s="37" t="n"/>
+      <c r="K22" s="37" t="n"/>
+      <c r="L22" s="37" t="n"/>
+      <c r="M22" s="37" t="n"/>
       <c r="N22" s="4" t="n"/>
       <c r="O22" s="4" t="n"/>
-      <c r="P22" s="14">
+      <c r="P22" s="36">
         <f>IF(A22="","",N(H22)+SUM(I22:M22))</f>
         <v/>
       </c>
@@ -1077,25 +1100,25 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="n"/>
+      <c r="A23" s="35" t="n"/>
       <c r="B23" s="4" t="n"/>
       <c r="C23" s="4" t="n"/>
       <c r="D23" s="4" t="n"/>
       <c r="E23" s="4" t="n"/>
       <c r="F23" s="4" t="n"/>
       <c r="G23" s="4" t="n"/>
-      <c r="H23" s="14">
+      <c r="H23" s="36">
         <f>IF(G23="","",G23*$C$11)</f>
         <v/>
       </c>
-      <c r="I23" s="15" t="n"/>
-      <c r="J23" s="15" t="n"/>
-      <c r="K23" s="15" t="n"/>
-      <c r="L23" s="15" t="n"/>
-      <c r="M23" s="15" t="n"/>
+      <c r="I23" s="37" t="n"/>
+      <c r="J23" s="37" t="n"/>
+      <c r="K23" s="37" t="n"/>
+      <c r="L23" s="37" t="n"/>
+      <c r="M23" s="37" t="n"/>
       <c r="N23" s="4" t="n"/>
       <c r="O23" s="4" t="n"/>
-      <c r="P23" s="14">
+      <c r="P23" s="36">
         <f>IF(A23="","",N(H23)+SUM(I23:M23))</f>
         <v/>
       </c>
@@ -1105,25 +1128,25 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="n"/>
+      <c r="A24" s="35" t="n"/>
       <c r="B24" s="4" t="n"/>
       <c r="C24" s="4" t="n"/>
       <c r="D24" s="4" t="n"/>
       <c r="E24" s="4" t="n"/>
       <c r="F24" s="4" t="n"/>
       <c r="G24" s="4" t="n"/>
-      <c r="H24" s="14">
+      <c r="H24" s="36">
         <f>IF(G24="","",G24*$C$11)</f>
         <v/>
       </c>
-      <c r="I24" s="15" t="n"/>
-      <c r="J24" s="15" t="n"/>
-      <c r="K24" s="15" t="n"/>
-      <c r="L24" s="15" t="n"/>
-      <c r="M24" s="15" t="n"/>
+      <c r="I24" s="37" t="n"/>
+      <c r="J24" s="37" t="n"/>
+      <c r="K24" s="37" t="n"/>
+      <c r="L24" s="37" t="n"/>
+      <c r="M24" s="37" t="n"/>
       <c r="N24" s="4" t="n"/>
       <c r="O24" s="4" t="n"/>
-      <c r="P24" s="14">
+      <c r="P24" s="36">
         <f>IF(A24="","",N(H24)+SUM(I24:M24))</f>
         <v/>
       </c>
@@ -1133,25 +1156,25 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="n"/>
+      <c r="A25" s="35" t="n"/>
       <c r="B25" s="4" t="n"/>
       <c r="C25" s="4" t="n"/>
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="n"/>
       <c r="G25" s="4" t="n"/>
-      <c r="H25" s="14">
+      <c r="H25" s="36">
         <f>IF(G25="","",G25*$C$11)</f>
         <v/>
       </c>
-      <c r="I25" s="15" t="n"/>
-      <c r="J25" s="15" t="n"/>
-      <c r="K25" s="15" t="n"/>
-      <c r="L25" s="15" t="n"/>
-      <c r="M25" s="15" t="n"/>
+      <c r="I25" s="37" t="n"/>
+      <c r="J25" s="37" t="n"/>
+      <c r="K25" s="37" t="n"/>
+      <c r="L25" s="37" t="n"/>
+      <c r="M25" s="37" t="n"/>
       <c r="N25" s="4" t="n"/>
       <c r="O25" s="4" t="n"/>
-      <c r="P25" s="14">
+      <c r="P25" s="36">
         <f>IF(A25="","",N(H25)+SUM(I25:M25))</f>
         <v/>
       </c>
@@ -1161,25 +1184,25 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="n"/>
+      <c r="A26" s="35" t="n"/>
       <c r="B26" s="4" t="n"/>
       <c r="C26" s="4" t="n"/>
       <c r="D26" s="4" t="n"/>
       <c r="E26" s="4" t="n"/>
       <c r="F26" s="4" t="n"/>
       <c r="G26" s="4" t="n"/>
-      <c r="H26" s="14">
+      <c r="H26" s="36">
         <f>IF(G26="","",G26*$C$11)</f>
         <v/>
       </c>
-      <c r="I26" s="15" t="n"/>
-      <c r="J26" s="15" t="n"/>
-      <c r="K26" s="15" t="n"/>
-      <c r="L26" s="15" t="n"/>
-      <c r="M26" s="15" t="n"/>
+      <c r="I26" s="37" t="n"/>
+      <c r="J26" s="37" t="n"/>
+      <c r="K26" s="37" t="n"/>
+      <c r="L26" s="37" t="n"/>
+      <c r="M26" s="37" t="n"/>
       <c r="N26" s="4" t="n"/>
       <c r="O26" s="4" t="n"/>
-      <c r="P26" s="14">
+      <c r="P26" s="36">
         <f>IF(A26="","",N(H26)+SUM(I26:M26))</f>
         <v/>
       </c>
@@ -1189,25 +1212,25 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="n"/>
+      <c r="A27" s="35" t="n"/>
       <c r="B27" s="4" t="n"/>
       <c r="C27" s="4" t="n"/>
       <c r="D27" s="4" t="n"/>
       <c r="E27" s="4" t="n"/>
       <c r="F27" s="4" t="n"/>
       <c r="G27" s="4" t="n"/>
-      <c r="H27" s="14">
+      <c r="H27" s="36">
         <f>IF(G27="","",G27*$C$11)</f>
         <v/>
       </c>
-      <c r="I27" s="15" t="n"/>
-      <c r="J27" s="15" t="n"/>
-      <c r="K27" s="15" t="n"/>
-      <c r="L27" s="15" t="n"/>
-      <c r="M27" s="15" t="n"/>
+      <c r="I27" s="37" t="n"/>
+      <c r="J27" s="37" t="n"/>
+      <c r="K27" s="37" t="n"/>
+      <c r="L27" s="37" t="n"/>
+      <c r="M27" s="37" t="n"/>
       <c r="N27" s="4" t="n"/>
       <c r="O27" s="4" t="n"/>
-      <c r="P27" s="14">
+      <c r="P27" s="36">
         <f>IF(A27="","",N(H27)+SUM(I27:M27))</f>
         <v/>
       </c>
@@ -1217,25 +1240,25 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="n"/>
+      <c r="A28" s="35" t="n"/>
       <c r="B28" s="4" t="n"/>
       <c r="C28" s="4" t="n"/>
       <c r="D28" s="4" t="n"/>
       <c r="E28" s="4" t="n"/>
       <c r="F28" s="4" t="n"/>
       <c r="G28" s="4" t="n"/>
-      <c r="H28" s="14">
+      <c r="H28" s="36">
         <f>IF(G28="","",G28*$C$11)</f>
         <v/>
       </c>
-      <c r="I28" s="15" t="n"/>
-      <c r="J28" s="15" t="n"/>
-      <c r="K28" s="15" t="n"/>
-      <c r="L28" s="15" t="n"/>
-      <c r="M28" s="15" t="n"/>
+      <c r="I28" s="37" t="n"/>
+      <c r="J28" s="37" t="n"/>
+      <c r="K28" s="37" t="n"/>
+      <c r="L28" s="37" t="n"/>
+      <c r="M28" s="37" t="n"/>
       <c r="N28" s="4" t="n"/>
       <c r="O28" s="4" t="n"/>
-      <c r="P28" s="14">
+      <c r="P28" s="36">
         <f>IF(A28="","",N(H28)+SUM(I28:M28))</f>
         <v/>
       </c>
@@ -1245,25 +1268,25 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="n"/>
+      <c r="A29" s="35" t="n"/>
       <c r="B29" s="4" t="n"/>
       <c r="C29" s="4" t="n"/>
       <c r="D29" s="4" t="n"/>
       <c r="E29" s="4" t="n"/>
       <c r="F29" s="4" t="n"/>
       <c r="G29" s="4" t="n"/>
-      <c r="H29" s="14">
+      <c r="H29" s="36">
         <f>IF(G29="","",G29*$C$11)</f>
         <v/>
       </c>
-      <c r="I29" s="15" t="n"/>
-      <c r="J29" s="15" t="n"/>
-      <c r="K29" s="15" t="n"/>
-      <c r="L29" s="15" t="n"/>
-      <c r="M29" s="15" t="n"/>
+      <c r="I29" s="37" t="n"/>
+      <c r="J29" s="37" t="n"/>
+      <c r="K29" s="37" t="n"/>
+      <c r="L29" s="37" t="n"/>
+      <c r="M29" s="37" t="n"/>
       <c r="N29" s="4" t="n"/>
       <c r="O29" s="4" t="n"/>
-      <c r="P29" s="14">
+      <c r="P29" s="36">
         <f>IF(A29="","",N(H29)+SUM(I29:M29))</f>
         <v/>
       </c>
@@ -1273,25 +1296,25 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="n"/>
+      <c r="A30" s="35" t="n"/>
       <c r="B30" s="4" t="n"/>
       <c r="C30" s="4" t="n"/>
       <c r="D30" s="4" t="n"/>
       <c r="E30" s="4" t="n"/>
       <c r="F30" s="4" t="n"/>
       <c r="G30" s="4" t="n"/>
-      <c r="H30" s="14">
+      <c r="H30" s="36">
         <f>IF(G30="","",G30*$C$11)</f>
         <v/>
       </c>
-      <c r="I30" s="15" t="n"/>
-      <c r="J30" s="15" t="n"/>
-      <c r="K30" s="15" t="n"/>
-      <c r="L30" s="15" t="n"/>
-      <c r="M30" s="15" t="n"/>
+      <c r="I30" s="37" t="n"/>
+      <c r="J30" s="37" t="n"/>
+      <c r="K30" s="37" t="n"/>
+      <c r="L30" s="37" t="n"/>
+      <c r="M30" s="37" t="n"/>
       <c r="N30" s="4" t="n"/>
       <c r="O30" s="4" t="n"/>
-      <c r="P30" s="14">
+      <c r="P30" s="36">
         <f>IF(A30="","",N(H30)+SUM(I30:M30))</f>
         <v/>
       </c>
@@ -1301,25 +1324,25 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="n"/>
+      <c r="A31" s="35" t="n"/>
       <c r="B31" s="4" t="n"/>
       <c r="C31" s="4" t="n"/>
       <c r="D31" s="4" t="n"/>
       <c r="E31" s="4" t="n"/>
       <c r="F31" s="4" t="n"/>
       <c r="G31" s="4" t="n"/>
-      <c r="H31" s="14">
+      <c r="H31" s="36">
         <f>IF(G31="","",G31*$C$11)</f>
         <v/>
       </c>
-      <c r="I31" s="15" t="n"/>
-      <c r="J31" s="15" t="n"/>
-      <c r="K31" s="15" t="n"/>
-      <c r="L31" s="15" t="n"/>
-      <c r="M31" s="15" t="n"/>
+      <c r="I31" s="37" t="n"/>
+      <c r="J31" s="37" t="n"/>
+      <c r="K31" s="37" t="n"/>
+      <c r="L31" s="37" t="n"/>
+      <c r="M31" s="37" t="n"/>
       <c r="N31" s="4" t="n"/>
       <c r="O31" s="4" t="n"/>
-      <c r="P31" s="14">
+      <c r="P31" s="36">
         <f>IF(A31="","",N(H31)+SUM(I31:M31))</f>
         <v/>
       </c>
@@ -1329,25 +1352,25 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="n"/>
+      <c r="A32" s="35" t="n"/>
       <c r="B32" s="4" t="n"/>
       <c r="C32" s="4" t="n"/>
       <c r="D32" s="4" t="n"/>
       <c r="E32" s="4" t="n"/>
       <c r="F32" s="4" t="n"/>
       <c r="G32" s="4" t="n"/>
-      <c r="H32" s="14">
+      <c r="H32" s="36">
         <f>IF(G32="","",G32*$C$11)</f>
         <v/>
       </c>
-      <c r="I32" s="15" t="n"/>
-      <c r="J32" s="15" t="n"/>
-      <c r="K32" s="15" t="n"/>
-      <c r="L32" s="15" t="n"/>
-      <c r="M32" s="15" t="n"/>
+      <c r="I32" s="37" t="n"/>
+      <c r="J32" s="37" t="n"/>
+      <c r="K32" s="37" t="n"/>
+      <c r="L32" s="37" t="n"/>
+      <c r="M32" s="37" t="n"/>
       <c r="N32" s="4" t="n"/>
       <c r="O32" s="4" t="n"/>
-      <c r="P32" s="14">
+      <c r="P32" s="36">
         <f>IF(A32="","",N(H32)+SUM(I32:M32))</f>
         <v/>
       </c>
@@ -1357,25 +1380,25 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="n"/>
+      <c r="A33" s="35" t="n"/>
       <c r="B33" s="4" t="n"/>
       <c r="C33" s="4" t="n"/>
       <c r="D33" s="4" t="n"/>
       <c r="E33" s="4" t="n"/>
       <c r="F33" s="4" t="n"/>
       <c r="G33" s="4" t="n"/>
-      <c r="H33" s="14">
+      <c r="H33" s="36">
         <f>IF(G33="","",G33*$C$11)</f>
         <v/>
       </c>
-      <c r="I33" s="15" t="n"/>
-      <c r="J33" s="15" t="n"/>
-      <c r="K33" s="15" t="n"/>
-      <c r="L33" s="15" t="n"/>
-      <c r="M33" s="15" t="n"/>
+      <c r="I33" s="37" t="n"/>
+      <c r="J33" s="37" t="n"/>
+      <c r="K33" s="37" t="n"/>
+      <c r="L33" s="37" t="n"/>
+      <c r="M33" s="37" t="n"/>
       <c r="N33" s="4" t="n"/>
       <c r="O33" s="4" t="n"/>
-      <c r="P33" s="14">
+      <c r="P33" s="36">
         <f>IF(A33="","",N(H33)+SUM(I33:M33))</f>
         <v/>
       </c>
@@ -1385,25 +1408,25 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="n"/>
+      <c r="A34" s="35" t="n"/>
       <c r="B34" s="4" t="n"/>
       <c r="C34" s="4" t="n"/>
       <c r="D34" s="4" t="n"/>
       <c r="E34" s="4" t="n"/>
       <c r="F34" s="4" t="n"/>
       <c r="G34" s="4" t="n"/>
-      <c r="H34" s="14">
+      <c r="H34" s="36">
         <f>IF(G34="","",G34*$C$11)</f>
         <v/>
       </c>
-      <c r="I34" s="15" t="n"/>
-      <c r="J34" s="15" t="n"/>
-      <c r="K34" s="15" t="n"/>
-      <c r="L34" s="15" t="n"/>
-      <c r="M34" s="15" t="n"/>
+      <c r="I34" s="37" t="n"/>
+      <c r="J34" s="37" t="n"/>
+      <c r="K34" s="37" t="n"/>
+      <c r="L34" s="37" t="n"/>
+      <c r="M34" s="37" t="n"/>
       <c r="N34" s="4" t="n"/>
       <c r="O34" s="4" t="n"/>
-      <c r="P34" s="14">
+      <c r="P34" s="36">
         <f>IF(A34="","",N(H34)+SUM(I34:M34))</f>
         <v/>
       </c>
@@ -1413,25 +1436,25 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="n"/>
+      <c r="A35" s="35" t="n"/>
       <c r="B35" s="4" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="4" t="n"/>
       <c r="E35" s="4" t="n"/>
       <c r="F35" s="4" t="n"/>
       <c r="G35" s="4" t="n"/>
-      <c r="H35" s="14">
+      <c r="H35" s="36">
         <f>IF(G35="","",G35*$C$11)</f>
         <v/>
       </c>
-      <c r="I35" s="15" t="n"/>
-      <c r="J35" s="15" t="n"/>
-      <c r="K35" s="15" t="n"/>
-      <c r="L35" s="15" t="n"/>
-      <c r="M35" s="15" t="n"/>
+      <c r="I35" s="37" t="n"/>
+      <c r="J35" s="37" t="n"/>
+      <c r="K35" s="37" t="n"/>
+      <c r="L35" s="37" t="n"/>
+      <c r="M35" s="37" t="n"/>
       <c r="N35" s="4" t="n"/>
       <c r="O35" s="4" t="n"/>
-      <c r="P35" s="14">
+      <c r="P35" s="36">
         <f>IF(A35="","",N(H35)+SUM(I35:M35))</f>
         <v/>
       </c>
@@ -1441,25 +1464,25 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="13" t="n"/>
+      <c r="A36" s="35" t="n"/>
       <c r="B36" s="4" t="n"/>
       <c r="C36" s="4" t="n"/>
       <c r="D36" s="4" t="n"/>
       <c r="E36" s="4" t="n"/>
       <c r="F36" s="4" t="n"/>
       <c r="G36" s="4" t="n"/>
-      <c r="H36" s="14">
+      <c r="H36" s="36">
         <f>IF(G36="","",G36*$C$11)</f>
         <v/>
       </c>
-      <c r="I36" s="15" t="n"/>
-      <c r="J36" s="15" t="n"/>
-      <c r="K36" s="15" t="n"/>
-      <c r="L36" s="15" t="n"/>
-      <c r="M36" s="15" t="n"/>
+      <c r="I36" s="37" t="n"/>
+      <c r="J36" s="37" t="n"/>
+      <c r="K36" s="37" t="n"/>
+      <c r="L36" s="37" t="n"/>
+      <c r="M36" s="37" t="n"/>
       <c r="N36" s="4" t="n"/>
       <c r="O36" s="4" t="n"/>
-      <c r="P36" s="14">
+      <c r="P36" s="36">
         <f>IF(A36="","",N(H36)+SUM(I36:M36))</f>
         <v/>
       </c>
@@ -1469,25 +1492,25 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="n"/>
+      <c r="A37" s="35" t="n"/>
       <c r="B37" s="4" t="n"/>
       <c r="C37" s="4" t="n"/>
       <c r="D37" s="4" t="n"/>
       <c r="E37" s="4" t="n"/>
       <c r="F37" s="4" t="n"/>
       <c r="G37" s="4" t="n"/>
-      <c r="H37" s="14">
+      <c r="H37" s="36">
         <f>IF(G37="","",G37*$C$11)</f>
         <v/>
       </c>
-      <c r="I37" s="15" t="n"/>
-      <c r="J37" s="15" t="n"/>
-      <c r="K37" s="15" t="n"/>
-      <c r="L37" s="15" t="n"/>
-      <c r="M37" s="15" t="n"/>
+      <c r="I37" s="37" t="n"/>
+      <c r="J37" s="37" t="n"/>
+      <c r="K37" s="37" t="n"/>
+      <c r="L37" s="37" t="n"/>
+      <c r="M37" s="37" t="n"/>
       <c r="N37" s="4" t="n"/>
       <c r="O37" s="4" t="n"/>
-      <c r="P37" s="14">
+      <c r="P37" s="36">
         <f>IF(A37="","",N(H37)+SUM(I37:M37))</f>
         <v/>
       </c>
@@ -1497,25 +1520,25 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="n"/>
+      <c r="A38" s="35" t="n"/>
       <c r="B38" s="4" t="n"/>
       <c r="C38" s="4" t="n"/>
       <c r="D38" s="4" t="n"/>
       <c r="E38" s="4" t="n"/>
       <c r="F38" s="4" t="n"/>
       <c r="G38" s="4" t="n"/>
-      <c r="H38" s="14">
+      <c r="H38" s="36">
         <f>IF(G38="","",G38*$C$11)</f>
         <v/>
       </c>
-      <c r="I38" s="15" t="n"/>
-      <c r="J38" s="15" t="n"/>
-      <c r="K38" s="15" t="n"/>
-      <c r="L38" s="15" t="n"/>
-      <c r="M38" s="15" t="n"/>
+      <c r="I38" s="37" t="n"/>
+      <c r="J38" s="37" t="n"/>
+      <c r="K38" s="37" t="n"/>
+      <c r="L38" s="37" t="n"/>
+      <c r="M38" s="37" t="n"/>
       <c r="N38" s="4" t="n"/>
       <c r="O38" s="4" t="n"/>
-      <c r="P38" s="14">
+      <c r="P38" s="36">
         <f>IF(A38="","",N(H38)+SUM(I38:M38))</f>
         <v/>
       </c>
@@ -1525,25 +1548,25 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="13" t="n"/>
+      <c r="A39" s="35" t="n"/>
       <c r="B39" s="4" t="n"/>
       <c r="C39" s="4" t="n"/>
       <c r="D39" s="4" t="n"/>
       <c r="E39" s="4" t="n"/>
       <c r="F39" s="4" t="n"/>
       <c r="G39" s="4" t="n"/>
-      <c r="H39" s="14">
+      <c r="H39" s="36">
         <f>IF(G39="","",G39*$C$11)</f>
         <v/>
       </c>
-      <c r="I39" s="15" t="n"/>
-      <c r="J39" s="15" t="n"/>
-      <c r="K39" s="15" t="n"/>
-      <c r="L39" s="15" t="n"/>
-      <c r="M39" s="15" t="n"/>
+      <c r="I39" s="37" t="n"/>
+      <c r="J39" s="37" t="n"/>
+      <c r="K39" s="37" t="n"/>
+      <c r="L39" s="37" t="n"/>
+      <c r="M39" s="37" t="n"/>
       <c r="N39" s="4" t="n"/>
       <c r="O39" s="4" t="n"/>
-      <c r="P39" s="14">
+      <c r="P39" s="36">
         <f>IF(A39="","",N(H39)+SUM(I39:M39))</f>
         <v/>
       </c>
@@ -1553,25 +1576,25 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="13" t="n"/>
+      <c r="A40" s="35" t="n"/>
       <c r="B40" s="4" t="n"/>
       <c r="C40" s="4" t="n"/>
       <c r="D40" s="4" t="n"/>
       <c r="E40" s="4" t="n"/>
       <c r="F40" s="4" t="n"/>
       <c r="G40" s="4" t="n"/>
-      <c r="H40" s="14">
+      <c r="H40" s="36">
         <f>IF(G40="","",G40*$C$11)</f>
         <v/>
       </c>
-      <c r="I40" s="15" t="n"/>
-      <c r="J40" s="15" t="n"/>
-      <c r="K40" s="15" t="n"/>
-      <c r="L40" s="15" t="n"/>
-      <c r="M40" s="15" t="n"/>
+      <c r="I40" s="37" t="n"/>
+      <c r="J40" s="37" t="n"/>
+      <c r="K40" s="37" t="n"/>
+      <c r="L40" s="37" t="n"/>
+      <c r="M40" s="37" t="n"/>
       <c r="N40" s="4" t="n"/>
       <c r="O40" s="4" t="n"/>
-      <c r="P40" s="14">
+      <c r="P40" s="36">
         <f>IF(A40="","",N(H40)+SUM(I40:M40))</f>
         <v/>
       </c>
@@ -1580,7 +1603,6 @@
         <v/>
       </c>
     </row>
-    <row r="41"/>
     <row r="42">
       <c r="F42" s="3" t="inlineStr">
         <is>
@@ -1591,31 +1613,31 @@
         <f>SUM(G16:G40)</f>
         <v/>
       </c>
-      <c r="H42" s="18">
+      <c r="H42" s="38">
         <f>SUM(H16:H40)</f>
         <v/>
       </c>
-      <c r="I42" s="18">
+      <c r="I42" s="38">
         <f>SUM(I16:I40)</f>
         <v/>
       </c>
-      <c r="J42" s="18">
+      <c r="J42" s="38">
         <f>SUM(J16:J40)</f>
         <v/>
       </c>
-      <c r="K42" s="18">
+      <c r="K42" s="38">
         <f>SUM(K16:K40)</f>
         <v/>
       </c>
-      <c r="L42" s="18">
+      <c r="L42" s="38">
         <f>SUM(L16:L40)</f>
         <v/>
       </c>
-      <c r="M42" s="18">
+      <c r="M42" s="38">
         <f>SUM(M16:M40)</f>
         <v/>
       </c>
-      <c r="P42" s="18">
+      <c r="P42" s="38">
         <f>SUM(P16:P40)</f>
         <v/>
       </c>
@@ -1626,7 +1648,7 @@
           <t>TOTALE RIMBORSABILE (solo righe OK)</t>
         </is>
       </c>
-      <c r="P43" s="19">
+      <c r="P43" s="39">
         <f>SUMIFS(P16:P40,Q16:Q40,"OK")</f>
         <v/>
       </c>
@@ -1642,8 +1664,6 @@
         <v/>
       </c>
     </row>
-    <row r="45"/>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
@@ -1656,7 +1676,6 @@
       <c r="F47" s="21" t="n"/>
       <c r="G47" s="21" t="n"/>
     </row>
-    <row r="48"/>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
@@ -1669,7 +1688,6 @@
       <c r="F49" s="21" t="n"/>
       <c r="G49" s="21" t="n"/>
     </row>
-    <row r="50"/>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
@@ -1682,7 +1700,6 @@
       <c r="F51" s="21" t="n"/>
       <c r="G51" s="21" t="n"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
@@ -1767,7 +1784,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1785,7 +1801,7 @@
           <t>Mese di riferimento</t>
         </is>
       </c>
-      <c r="C5" s="23">
+      <c r="C5" s="40">
         <f>'Nota spese'!C6</f>
         <v/>
       </c>
@@ -1807,7 +1823,7 @@
           <t>Tariffa ACI €/km del veicolo</t>
         </is>
       </c>
-      <c r="C7" s="24">
+      <c r="C7" s="41">
         <f>'Nota spese'!C11</f>
         <v/>
       </c>
@@ -1818,7 +1834,7 @@
           <t>Indennità giornaliera da regolamento (€)</t>
         </is>
       </c>
-      <c r="C8" s="15" t="n">
+      <c r="C8" s="37" t="n">
         <v>46.48</v>
       </c>
     </row>
@@ -1828,7 +1844,7 @@
           <t>Soglia esente: nessun rimborso vitto/alloggio (€)</t>
         </is>
       </c>
-      <c r="C9" s="25" t="n">
+      <c r="C9" s="42" t="n">
         <v>46.48</v>
       </c>
       <c r="D9" s="26" t="inlineStr">
@@ -1843,7 +1859,7 @@
           <t>Soglia esente: rimborsato vitto OPPURE alloggio (€)</t>
         </is>
       </c>
-      <c r="C10" s="25" t="n">
+      <c r="C10" s="42" t="n">
         <v>30.99</v>
       </c>
     </row>
@@ -1853,7 +1869,7 @@
           <t>Soglia esente: rimborsati vitto E alloggio (€)</t>
         </is>
       </c>
-      <c r="C11" s="25" t="n">
+      <c r="C11" s="42" t="n">
         <v>15.49</v>
       </c>
     </row>
@@ -1868,7 +1884,6 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
@@ -1967,7 +1982,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="n">
+      <c r="A15" s="32" t="n">
         <v>46093</v>
       </c>
       <c r="B15" s="9" t="inlineStr">
@@ -1998,39 +2013,39 @@
       <c r="G15" s="9" t="n">
         <v>150</v>
       </c>
-      <c r="H15" s="10">
+      <c r="H15" s="33">
         <f>IF(G15="","",G15*$C$7)</f>
         <v/>
       </c>
-      <c r="I15" s="11" t="n">
+      <c r="I15" s="34" t="n">
         <v>10.4</v>
       </c>
-      <c r="J15" s="11" t="n">
+      <c r="J15" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="K15" s="11" t="n">
+      <c r="K15" s="34" t="n">
         <v>0</v>
       </c>
-      <c r="L15" s="11" t="n">
+      <c r="L15" s="34" t="n">
         <v>0</v>
       </c>
       <c r="M15" s="9" t="n"/>
-      <c r="N15" s="10">
+      <c r="N15" s="33">
         <f>IF(A15="","",IF(COUNTIF($A$15:A15,A15)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O15" s="10">
+      <c r="O15" s="33">
         <f>IF(A15="","",MIN(N15,IF(AND(SUMIF($A$15:$A$39,A15,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A15,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A15,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A15,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P15" s="10">
+      <c r="P15" s="33">
         <f>IF(A15="","",N15-O15)</f>
         <v/>
       </c>
       <c r="Q15" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="R15" s="10">
+      <c r="R15" s="33">
         <f>IF(A15="","",N(H15)+N(I15)+N(J15)+N(K15)+N(L15)+N15)</f>
         <v/>
       </c>
@@ -2040,36 +2055,36 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="n"/>
+      <c r="A16" s="35" t="n"/>
       <c r="B16" s="4" t="n"/>
       <c r="C16" s="4" t="n"/>
       <c r="D16" s="4" t="n"/>
       <c r="E16" s="4" t="n"/>
       <c r="F16" s="4" t="n"/>
       <c r="G16" s="4" t="n"/>
-      <c r="H16" s="14">
+      <c r="H16" s="36">
         <f>IF(G16="","",G16*$C$7)</f>
         <v/>
       </c>
-      <c r="I16" s="15" t="n"/>
-      <c r="J16" s="15" t="n"/>
-      <c r="K16" s="15" t="n"/>
-      <c r="L16" s="15" t="n"/>
+      <c r="I16" s="37" t="n"/>
+      <c r="J16" s="37" t="n"/>
+      <c r="K16" s="37" t="n"/>
+      <c r="L16" s="37" t="n"/>
       <c r="M16" s="4" t="n"/>
-      <c r="N16" s="14">
+      <c r="N16" s="36">
         <f>IF(A16="","",IF(COUNTIF($A$15:A16,A16)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O16" s="14">
+      <c r="O16" s="36">
         <f>IF(A16="","",MIN(N16,IF(AND(SUMIF($A$15:$A$39,A16,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A16,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A16,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A16,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P16" s="14">
+      <c r="P16" s="36">
         <f>IF(A16="","",N16-O16)</f>
         <v/>
       </c>
       <c r="Q16" s="4" t="n"/>
-      <c r="R16" s="14">
+      <c r="R16" s="36">
         <f>IF(A16="","",N(H16)+N(I16)+N(J16)+N(K16)+N(L16)+N16)</f>
         <v/>
       </c>
@@ -2079,36 +2094,36 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="n"/>
+      <c r="A17" s="35" t="n"/>
       <c r="B17" s="4" t="n"/>
       <c r="C17" s="4" t="n"/>
       <c r="D17" s="4" t="n"/>
       <c r="E17" s="4" t="n"/>
       <c r="F17" s="4" t="n"/>
       <c r="G17" s="4" t="n"/>
-      <c r="H17" s="14">
+      <c r="H17" s="36">
         <f>IF(G17="","",G17*$C$7)</f>
         <v/>
       </c>
-      <c r="I17" s="15" t="n"/>
-      <c r="J17" s="15" t="n"/>
-      <c r="K17" s="15" t="n"/>
-      <c r="L17" s="15" t="n"/>
+      <c r="I17" s="37" t="n"/>
+      <c r="J17" s="37" t="n"/>
+      <c r="K17" s="37" t="n"/>
+      <c r="L17" s="37" t="n"/>
       <c r="M17" s="4" t="n"/>
-      <c r="N17" s="14">
+      <c r="N17" s="36">
         <f>IF(A17="","",IF(COUNTIF($A$15:A17,A17)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O17" s="14">
+      <c r="O17" s="36">
         <f>IF(A17="","",MIN(N17,IF(AND(SUMIF($A$15:$A$39,A17,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A17,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A17,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A17,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P17" s="14">
+      <c r="P17" s="36">
         <f>IF(A17="","",N17-O17)</f>
         <v/>
       </c>
       <c r="Q17" s="4" t="n"/>
-      <c r="R17" s="14">
+      <c r="R17" s="36">
         <f>IF(A17="","",N(H17)+N(I17)+N(J17)+N(K17)+N(L17)+N17)</f>
         <v/>
       </c>
@@ -2118,36 +2133,36 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="n"/>
+      <c r="A18" s="35" t="n"/>
       <c r="B18" s="4" t="n"/>
       <c r="C18" s="4" t="n"/>
       <c r="D18" s="4" t="n"/>
       <c r="E18" s="4" t="n"/>
       <c r="F18" s="4" t="n"/>
       <c r="G18" s="4" t="n"/>
-      <c r="H18" s="14">
+      <c r="H18" s="36">
         <f>IF(G18="","",G18*$C$7)</f>
         <v/>
       </c>
-      <c r="I18" s="15" t="n"/>
-      <c r="J18" s="15" t="n"/>
-      <c r="K18" s="15" t="n"/>
-      <c r="L18" s="15" t="n"/>
+      <c r="I18" s="37" t="n"/>
+      <c r="J18" s="37" t="n"/>
+      <c r="K18" s="37" t="n"/>
+      <c r="L18" s="37" t="n"/>
       <c r="M18" s="4" t="n"/>
-      <c r="N18" s="14">
+      <c r="N18" s="36">
         <f>IF(A18="","",IF(COUNTIF($A$15:A18,A18)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O18" s="14">
+      <c r="O18" s="36">
         <f>IF(A18="","",MIN(N18,IF(AND(SUMIF($A$15:$A$39,A18,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A18,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A18,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A18,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P18" s="14">
+      <c r="P18" s="36">
         <f>IF(A18="","",N18-O18)</f>
         <v/>
       </c>
       <c r="Q18" s="4" t="n"/>
-      <c r="R18" s="14">
+      <c r="R18" s="36">
         <f>IF(A18="","",N(H18)+N(I18)+N(J18)+N(K18)+N(L18)+N18)</f>
         <v/>
       </c>
@@ -2157,36 +2172,36 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="n"/>
+      <c r="A19" s="35" t="n"/>
       <c r="B19" s="4" t="n"/>
       <c r="C19" s="4" t="n"/>
       <c r="D19" s="4" t="n"/>
       <c r="E19" s="4" t="n"/>
       <c r="F19" s="4" t="n"/>
       <c r="G19" s="4" t="n"/>
-      <c r="H19" s="14">
+      <c r="H19" s="36">
         <f>IF(G19="","",G19*$C$7)</f>
         <v/>
       </c>
-      <c r="I19" s="15" t="n"/>
-      <c r="J19" s="15" t="n"/>
-      <c r="K19" s="15" t="n"/>
-      <c r="L19" s="15" t="n"/>
+      <c r="I19" s="37" t="n"/>
+      <c r="J19" s="37" t="n"/>
+      <c r="K19" s="37" t="n"/>
+      <c r="L19" s="37" t="n"/>
       <c r="M19" s="4" t="n"/>
-      <c r="N19" s="14">
+      <c r="N19" s="36">
         <f>IF(A19="","",IF(COUNTIF($A$15:A19,A19)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O19" s="14">
+      <c r="O19" s="36">
         <f>IF(A19="","",MIN(N19,IF(AND(SUMIF($A$15:$A$39,A19,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A19,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A19,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A19,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P19" s="14">
+      <c r="P19" s="36">
         <f>IF(A19="","",N19-O19)</f>
         <v/>
       </c>
       <c r="Q19" s="4" t="n"/>
-      <c r="R19" s="14">
+      <c r="R19" s="36">
         <f>IF(A19="","",N(H19)+N(I19)+N(J19)+N(K19)+N(L19)+N19)</f>
         <v/>
       </c>
@@ -2196,36 +2211,36 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="n"/>
+      <c r="A20" s="35" t="n"/>
       <c r="B20" s="4" t="n"/>
       <c r="C20" s="4" t="n"/>
       <c r="D20" s="4" t="n"/>
       <c r="E20" s="4" t="n"/>
       <c r="F20" s="4" t="n"/>
       <c r="G20" s="4" t="n"/>
-      <c r="H20" s="14">
+      <c r="H20" s="36">
         <f>IF(G20="","",G20*$C$7)</f>
         <v/>
       </c>
-      <c r="I20" s="15" t="n"/>
-      <c r="J20" s="15" t="n"/>
-      <c r="K20" s="15" t="n"/>
-      <c r="L20" s="15" t="n"/>
+      <c r="I20" s="37" t="n"/>
+      <c r="J20" s="37" t="n"/>
+      <c r="K20" s="37" t="n"/>
+      <c r="L20" s="37" t="n"/>
       <c r="M20" s="4" t="n"/>
-      <c r="N20" s="14">
+      <c r="N20" s="36">
         <f>IF(A20="","",IF(COUNTIF($A$15:A20,A20)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O20" s="14">
+      <c r="O20" s="36">
         <f>IF(A20="","",MIN(N20,IF(AND(SUMIF($A$15:$A$39,A20,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A20,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A20,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A20,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P20" s="14">
+      <c r="P20" s="36">
         <f>IF(A20="","",N20-O20)</f>
         <v/>
       </c>
       <c r="Q20" s="4" t="n"/>
-      <c r="R20" s="14">
+      <c r="R20" s="36">
         <f>IF(A20="","",N(H20)+N(I20)+N(J20)+N(K20)+N(L20)+N20)</f>
         <v/>
       </c>
@@ -2235,36 +2250,36 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="n"/>
+      <c r="A21" s="35" t="n"/>
       <c r="B21" s="4" t="n"/>
       <c r="C21" s="4" t="n"/>
       <c r="D21" s="4" t="n"/>
       <c r="E21" s="4" t="n"/>
       <c r="F21" s="4" t="n"/>
       <c r="G21" s="4" t="n"/>
-      <c r="H21" s="14">
+      <c r="H21" s="36">
         <f>IF(G21="","",G21*$C$7)</f>
         <v/>
       </c>
-      <c r="I21" s="15" t="n"/>
-      <c r="J21" s="15" t="n"/>
-      <c r="K21" s="15" t="n"/>
-      <c r="L21" s="15" t="n"/>
+      <c r="I21" s="37" t="n"/>
+      <c r="J21" s="37" t="n"/>
+      <c r="K21" s="37" t="n"/>
+      <c r="L21" s="37" t="n"/>
       <c r="M21" s="4" t="n"/>
-      <c r="N21" s="14">
+      <c r="N21" s="36">
         <f>IF(A21="","",IF(COUNTIF($A$15:A21,A21)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O21" s="14">
+      <c r="O21" s="36">
         <f>IF(A21="","",MIN(N21,IF(AND(SUMIF($A$15:$A$39,A21,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A21,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A21,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A21,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P21" s="14">
+      <c r="P21" s="36">
         <f>IF(A21="","",N21-O21)</f>
         <v/>
       </c>
       <c r="Q21" s="4" t="n"/>
-      <c r="R21" s="14">
+      <c r="R21" s="36">
         <f>IF(A21="","",N(H21)+N(I21)+N(J21)+N(K21)+N(L21)+N21)</f>
         <v/>
       </c>
@@ -2274,36 +2289,36 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="n"/>
+      <c r="A22" s="35" t="n"/>
       <c r="B22" s="4" t="n"/>
       <c r="C22" s="4" t="n"/>
       <c r="D22" s="4" t="n"/>
       <c r="E22" s="4" t="n"/>
       <c r="F22" s="4" t="n"/>
       <c r="G22" s="4" t="n"/>
-      <c r="H22" s="14">
+      <c r="H22" s="36">
         <f>IF(G22="","",G22*$C$7)</f>
         <v/>
       </c>
-      <c r="I22" s="15" t="n"/>
-      <c r="J22" s="15" t="n"/>
-      <c r="K22" s="15" t="n"/>
-      <c r="L22" s="15" t="n"/>
+      <c r="I22" s="37" t="n"/>
+      <c r="J22" s="37" t="n"/>
+      <c r="K22" s="37" t="n"/>
+      <c r="L22" s="37" t="n"/>
       <c r="M22" s="4" t="n"/>
-      <c r="N22" s="14">
+      <c r="N22" s="36">
         <f>IF(A22="","",IF(COUNTIF($A$15:A22,A22)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O22" s="14">
+      <c r="O22" s="36">
         <f>IF(A22="","",MIN(N22,IF(AND(SUMIF($A$15:$A$39,A22,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A22,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A22,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A22,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P22" s="14">
+      <c r="P22" s="36">
         <f>IF(A22="","",N22-O22)</f>
         <v/>
       </c>
       <c r="Q22" s="4" t="n"/>
-      <c r="R22" s="14">
+      <c r="R22" s="36">
         <f>IF(A22="","",N(H22)+N(I22)+N(J22)+N(K22)+N(L22)+N22)</f>
         <v/>
       </c>
@@ -2313,36 +2328,36 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="n"/>
+      <c r="A23" s="35" t="n"/>
       <c r="B23" s="4" t="n"/>
       <c r="C23" s="4" t="n"/>
       <c r="D23" s="4" t="n"/>
       <c r="E23" s="4" t="n"/>
       <c r="F23" s="4" t="n"/>
       <c r="G23" s="4" t="n"/>
-      <c r="H23" s="14">
+      <c r="H23" s="36">
         <f>IF(G23="","",G23*$C$7)</f>
         <v/>
       </c>
-      <c r="I23" s="15" t="n"/>
-      <c r="J23" s="15" t="n"/>
-      <c r="K23" s="15" t="n"/>
-      <c r="L23" s="15" t="n"/>
+      <c r="I23" s="37" t="n"/>
+      <c r="J23" s="37" t="n"/>
+      <c r="K23" s="37" t="n"/>
+      <c r="L23" s="37" t="n"/>
       <c r="M23" s="4" t="n"/>
-      <c r="N23" s="14">
+      <c r="N23" s="36">
         <f>IF(A23="","",IF(COUNTIF($A$15:A23,A23)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O23" s="14">
+      <c r="O23" s="36">
         <f>IF(A23="","",MIN(N23,IF(AND(SUMIF($A$15:$A$39,A23,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A23,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A23,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A23,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P23" s="14">
+      <c r="P23" s="36">
         <f>IF(A23="","",N23-O23)</f>
         <v/>
       </c>
       <c r="Q23" s="4" t="n"/>
-      <c r="R23" s="14">
+      <c r="R23" s="36">
         <f>IF(A23="","",N(H23)+N(I23)+N(J23)+N(K23)+N(L23)+N23)</f>
         <v/>
       </c>
@@ -2352,36 +2367,36 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="n"/>
+      <c r="A24" s="35" t="n"/>
       <c r="B24" s="4" t="n"/>
       <c r="C24" s="4" t="n"/>
       <c r="D24" s="4" t="n"/>
       <c r="E24" s="4" t="n"/>
       <c r="F24" s="4" t="n"/>
       <c r="G24" s="4" t="n"/>
-      <c r="H24" s="14">
+      <c r="H24" s="36">
         <f>IF(G24="","",G24*$C$7)</f>
         <v/>
       </c>
-      <c r="I24" s="15" t="n"/>
-      <c r="J24" s="15" t="n"/>
-      <c r="K24" s="15" t="n"/>
-      <c r="L24" s="15" t="n"/>
+      <c r="I24" s="37" t="n"/>
+      <c r="J24" s="37" t="n"/>
+      <c r="K24" s="37" t="n"/>
+      <c r="L24" s="37" t="n"/>
       <c r="M24" s="4" t="n"/>
-      <c r="N24" s="14">
+      <c r="N24" s="36">
         <f>IF(A24="","",IF(COUNTIF($A$15:A24,A24)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O24" s="14">
+      <c r="O24" s="36">
         <f>IF(A24="","",MIN(N24,IF(AND(SUMIF($A$15:$A$39,A24,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A24,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A24,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A24,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P24" s="14">
+      <c r="P24" s="36">
         <f>IF(A24="","",N24-O24)</f>
         <v/>
       </c>
       <c r="Q24" s="4" t="n"/>
-      <c r="R24" s="14">
+      <c r="R24" s="36">
         <f>IF(A24="","",N(H24)+N(I24)+N(J24)+N(K24)+N(L24)+N24)</f>
         <v/>
       </c>
@@ -2391,36 +2406,36 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="n"/>
+      <c r="A25" s="35" t="n"/>
       <c r="B25" s="4" t="n"/>
       <c r="C25" s="4" t="n"/>
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="4" t="n"/>
       <c r="F25" s="4" t="n"/>
       <c r="G25" s="4" t="n"/>
-      <c r="H25" s="14">
+      <c r="H25" s="36">
         <f>IF(G25="","",G25*$C$7)</f>
         <v/>
       </c>
-      <c r="I25" s="15" t="n"/>
-      <c r="J25" s="15" t="n"/>
-      <c r="K25" s="15" t="n"/>
-      <c r="L25" s="15" t="n"/>
+      <c r="I25" s="37" t="n"/>
+      <c r="J25" s="37" t="n"/>
+      <c r="K25" s="37" t="n"/>
+      <c r="L25" s="37" t="n"/>
       <c r="M25" s="4" t="n"/>
-      <c r="N25" s="14">
+      <c r="N25" s="36">
         <f>IF(A25="","",IF(COUNTIF($A$15:A25,A25)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O25" s="14">
+      <c r="O25" s="36">
         <f>IF(A25="","",MIN(N25,IF(AND(SUMIF($A$15:$A$39,A25,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A25,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A25,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A25,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P25" s="14">
+      <c r="P25" s="36">
         <f>IF(A25="","",N25-O25)</f>
         <v/>
       </c>
       <c r="Q25" s="4" t="n"/>
-      <c r="R25" s="14">
+      <c r="R25" s="36">
         <f>IF(A25="","",N(H25)+N(I25)+N(J25)+N(K25)+N(L25)+N25)</f>
         <v/>
       </c>
@@ -2430,36 +2445,36 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="n"/>
+      <c r="A26" s="35" t="n"/>
       <c r="B26" s="4" t="n"/>
       <c r="C26" s="4" t="n"/>
       <c r="D26" s="4" t="n"/>
       <c r="E26" s="4" t="n"/>
       <c r="F26" s="4" t="n"/>
       <c r="G26" s="4" t="n"/>
-      <c r="H26" s="14">
+      <c r="H26" s="36">
         <f>IF(G26="","",G26*$C$7)</f>
         <v/>
       </c>
-      <c r="I26" s="15" t="n"/>
-      <c r="J26" s="15" t="n"/>
-      <c r="K26" s="15" t="n"/>
-      <c r="L26" s="15" t="n"/>
+      <c r="I26" s="37" t="n"/>
+      <c r="J26" s="37" t="n"/>
+      <c r="K26" s="37" t="n"/>
+      <c r="L26" s="37" t="n"/>
       <c r="M26" s="4" t="n"/>
-      <c r="N26" s="14">
+      <c r="N26" s="36">
         <f>IF(A26="","",IF(COUNTIF($A$15:A26,A26)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O26" s="14">
+      <c r="O26" s="36">
         <f>IF(A26="","",MIN(N26,IF(AND(SUMIF($A$15:$A$39,A26,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A26,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A26,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A26,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P26" s="14">
+      <c r="P26" s="36">
         <f>IF(A26="","",N26-O26)</f>
         <v/>
       </c>
       <c r="Q26" s="4" t="n"/>
-      <c r="R26" s="14">
+      <c r="R26" s="36">
         <f>IF(A26="","",N(H26)+N(I26)+N(J26)+N(K26)+N(L26)+N26)</f>
         <v/>
       </c>
@@ -2469,36 +2484,36 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="n"/>
+      <c r="A27" s="35" t="n"/>
       <c r="B27" s="4" t="n"/>
       <c r="C27" s="4" t="n"/>
       <c r="D27" s="4" t="n"/>
       <c r="E27" s="4" t="n"/>
       <c r="F27" s="4" t="n"/>
       <c r="G27" s="4" t="n"/>
-      <c r="H27" s="14">
+      <c r="H27" s="36">
         <f>IF(G27="","",G27*$C$7)</f>
         <v/>
       </c>
-      <c r="I27" s="15" t="n"/>
-      <c r="J27" s="15" t="n"/>
-      <c r="K27" s="15" t="n"/>
-      <c r="L27" s="15" t="n"/>
+      <c r="I27" s="37" t="n"/>
+      <c r="J27" s="37" t="n"/>
+      <c r="K27" s="37" t="n"/>
+      <c r="L27" s="37" t="n"/>
       <c r="M27" s="4" t="n"/>
-      <c r="N27" s="14">
+      <c r="N27" s="36">
         <f>IF(A27="","",IF(COUNTIF($A$15:A27,A27)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O27" s="14">
+      <c r="O27" s="36">
         <f>IF(A27="","",MIN(N27,IF(AND(SUMIF($A$15:$A$39,A27,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A27,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A27,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A27,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P27" s="14">
+      <c r="P27" s="36">
         <f>IF(A27="","",N27-O27)</f>
         <v/>
       </c>
       <c r="Q27" s="4" t="n"/>
-      <c r="R27" s="14">
+      <c r="R27" s="36">
         <f>IF(A27="","",N(H27)+N(I27)+N(J27)+N(K27)+N(L27)+N27)</f>
         <v/>
       </c>
@@ -2508,36 +2523,36 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="n"/>
+      <c r="A28" s="35" t="n"/>
       <c r="B28" s="4" t="n"/>
       <c r="C28" s="4" t="n"/>
       <c r="D28" s="4" t="n"/>
       <c r="E28" s="4" t="n"/>
       <c r="F28" s="4" t="n"/>
       <c r="G28" s="4" t="n"/>
-      <c r="H28" s="14">
+      <c r="H28" s="36">
         <f>IF(G28="","",G28*$C$7)</f>
         <v/>
       </c>
-      <c r="I28" s="15" t="n"/>
-      <c r="J28" s="15" t="n"/>
-      <c r="K28" s="15" t="n"/>
-      <c r="L28" s="15" t="n"/>
+      <c r="I28" s="37" t="n"/>
+      <c r="J28" s="37" t="n"/>
+      <c r="K28" s="37" t="n"/>
+      <c r="L28" s="37" t="n"/>
       <c r="M28" s="4" t="n"/>
-      <c r="N28" s="14">
+      <c r="N28" s="36">
         <f>IF(A28="","",IF(COUNTIF($A$15:A28,A28)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O28" s="14">
+      <c r="O28" s="36">
         <f>IF(A28="","",MIN(N28,IF(AND(SUMIF($A$15:$A$39,A28,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A28,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A28,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A28,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P28" s="14">
+      <c r="P28" s="36">
         <f>IF(A28="","",N28-O28)</f>
         <v/>
       </c>
       <c r="Q28" s="4" t="n"/>
-      <c r="R28" s="14">
+      <c r="R28" s="36">
         <f>IF(A28="","",N(H28)+N(I28)+N(J28)+N(K28)+N(L28)+N28)</f>
         <v/>
       </c>
@@ -2547,36 +2562,36 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="n"/>
+      <c r="A29" s="35" t="n"/>
       <c r="B29" s="4" t="n"/>
       <c r="C29" s="4" t="n"/>
       <c r="D29" s="4" t="n"/>
       <c r="E29" s="4" t="n"/>
       <c r="F29" s="4" t="n"/>
       <c r="G29" s="4" t="n"/>
-      <c r="H29" s="14">
+      <c r="H29" s="36">
         <f>IF(G29="","",G29*$C$7)</f>
         <v/>
       </c>
-      <c r="I29" s="15" t="n"/>
-      <c r="J29" s="15" t="n"/>
-      <c r="K29" s="15" t="n"/>
-      <c r="L29" s="15" t="n"/>
+      <c r="I29" s="37" t="n"/>
+      <c r="J29" s="37" t="n"/>
+      <c r="K29" s="37" t="n"/>
+      <c r="L29" s="37" t="n"/>
       <c r="M29" s="4" t="n"/>
-      <c r="N29" s="14">
+      <c r="N29" s="36">
         <f>IF(A29="","",IF(COUNTIF($A$15:A29,A29)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O29" s="14">
+      <c r="O29" s="36">
         <f>IF(A29="","",MIN(N29,IF(AND(SUMIF($A$15:$A$39,A29,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A29,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A29,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A29,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P29" s="14">
+      <c r="P29" s="36">
         <f>IF(A29="","",N29-O29)</f>
         <v/>
       </c>
       <c r="Q29" s="4" t="n"/>
-      <c r="R29" s="14">
+      <c r="R29" s="36">
         <f>IF(A29="","",N(H29)+N(I29)+N(J29)+N(K29)+N(L29)+N29)</f>
         <v/>
       </c>
@@ -2586,36 +2601,36 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="n"/>
+      <c r="A30" s="35" t="n"/>
       <c r="B30" s="4" t="n"/>
       <c r="C30" s="4" t="n"/>
       <c r="D30" s="4" t="n"/>
       <c r="E30" s="4" t="n"/>
       <c r="F30" s="4" t="n"/>
       <c r="G30" s="4" t="n"/>
-      <c r="H30" s="14">
+      <c r="H30" s="36">
         <f>IF(G30="","",G30*$C$7)</f>
         <v/>
       </c>
-      <c r="I30" s="15" t="n"/>
-      <c r="J30" s="15" t="n"/>
-      <c r="K30" s="15" t="n"/>
-      <c r="L30" s="15" t="n"/>
+      <c r="I30" s="37" t="n"/>
+      <c r="J30" s="37" t="n"/>
+      <c r="K30" s="37" t="n"/>
+      <c r="L30" s="37" t="n"/>
       <c r="M30" s="4" t="n"/>
-      <c r="N30" s="14">
+      <c r="N30" s="36">
         <f>IF(A30="","",IF(COUNTIF($A$15:A30,A30)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O30" s="14">
+      <c r="O30" s="36">
         <f>IF(A30="","",MIN(N30,IF(AND(SUMIF($A$15:$A$39,A30,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A30,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A30,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A30,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P30" s="14">
+      <c r="P30" s="36">
         <f>IF(A30="","",N30-O30)</f>
         <v/>
       </c>
       <c r="Q30" s="4" t="n"/>
-      <c r="R30" s="14">
+      <c r="R30" s="36">
         <f>IF(A30="","",N(H30)+N(I30)+N(J30)+N(K30)+N(L30)+N30)</f>
         <v/>
       </c>
@@ -2625,36 +2640,36 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="n"/>
+      <c r="A31" s="35" t="n"/>
       <c r="B31" s="4" t="n"/>
       <c r="C31" s="4" t="n"/>
       <c r="D31" s="4" t="n"/>
       <c r="E31" s="4" t="n"/>
       <c r="F31" s="4" t="n"/>
       <c r="G31" s="4" t="n"/>
-      <c r="H31" s="14">
+      <c r="H31" s="36">
         <f>IF(G31="","",G31*$C$7)</f>
         <v/>
       </c>
-      <c r="I31" s="15" t="n"/>
-      <c r="J31" s="15" t="n"/>
-      <c r="K31" s="15" t="n"/>
-      <c r="L31" s="15" t="n"/>
+      <c r="I31" s="37" t="n"/>
+      <c r="J31" s="37" t="n"/>
+      <c r="K31" s="37" t="n"/>
+      <c r="L31" s="37" t="n"/>
       <c r="M31" s="4" t="n"/>
-      <c r="N31" s="14">
+      <c r="N31" s="36">
         <f>IF(A31="","",IF(COUNTIF($A$15:A31,A31)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O31" s="14">
+      <c r="O31" s="36">
         <f>IF(A31="","",MIN(N31,IF(AND(SUMIF($A$15:$A$39,A31,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A31,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A31,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A31,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P31" s="14">
+      <c r="P31" s="36">
         <f>IF(A31="","",N31-O31)</f>
         <v/>
       </c>
       <c r="Q31" s="4" t="n"/>
-      <c r="R31" s="14">
+      <c r="R31" s="36">
         <f>IF(A31="","",N(H31)+N(I31)+N(J31)+N(K31)+N(L31)+N31)</f>
         <v/>
       </c>
@@ -2664,36 +2679,36 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="n"/>
+      <c r="A32" s="35" t="n"/>
       <c r="B32" s="4" t="n"/>
       <c r="C32" s="4" t="n"/>
       <c r="D32" s="4" t="n"/>
       <c r="E32" s="4" t="n"/>
       <c r="F32" s="4" t="n"/>
       <c r="G32" s="4" t="n"/>
-      <c r="H32" s="14">
+      <c r="H32" s="36">
         <f>IF(G32="","",G32*$C$7)</f>
         <v/>
       </c>
-      <c r="I32" s="15" t="n"/>
-      <c r="J32" s="15" t="n"/>
-      <c r="K32" s="15" t="n"/>
-      <c r="L32" s="15" t="n"/>
+      <c r="I32" s="37" t="n"/>
+      <c r="J32" s="37" t="n"/>
+      <c r="K32" s="37" t="n"/>
+      <c r="L32" s="37" t="n"/>
       <c r="M32" s="4" t="n"/>
-      <c r="N32" s="14">
+      <c r="N32" s="36">
         <f>IF(A32="","",IF(COUNTIF($A$15:A32,A32)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O32" s="14">
+      <c r="O32" s="36">
         <f>IF(A32="","",MIN(N32,IF(AND(SUMIF($A$15:$A$39,A32,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A32,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A32,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A32,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P32" s="14">
+      <c r="P32" s="36">
         <f>IF(A32="","",N32-O32)</f>
         <v/>
       </c>
       <c r="Q32" s="4" t="n"/>
-      <c r="R32" s="14">
+      <c r="R32" s="36">
         <f>IF(A32="","",N(H32)+N(I32)+N(J32)+N(K32)+N(L32)+N32)</f>
         <v/>
       </c>
@@ -2703,36 +2718,36 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="n"/>
+      <c r="A33" s="35" t="n"/>
       <c r="B33" s="4" t="n"/>
       <c r="C33" s="4" t="n"/>
       <c r="D33" s="4" t="n"/>
       <c r="E33" s="4" t="n"/>
       <c r="F33" s="4" t="n"/>
       <c r="G33" s="4" t="n"/>
-      <c r="H33" s="14">
+      <c r="H33" s="36">
         <f>IF(G33="","",G33*$C$7)</f>
         <v/>
       </c>
-      <c r="I33" s="15" t="n"/>
-      <c r="J33" s="15" t="n"/>
-      <c r="K33" s="15" t="n"/>
-      <c r="L33" s="15" t="n"/>
+      <c r="I33" s="37" t="n"/>
+      <c r="J33" s="37" t="n"/>
+      <c r="K33" s="37" t="n"/>
+      <c r="L33" s="37" t="n"/>
       <c r="M33" s="4" t="n"/>
-      <c r="N33" s="14">
+      <c r="N33" s="36">
         <f>IF(A33="","",IF(COUNTIF($A$15:A33,A33)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O33" s="14">
+      <c r="O33" s="36">
         <f>IF(A33="","",MIN(N33,IF(AND(SUMIF($A$15:$A$39,A33,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A33,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A33,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A33,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P33" s="14">
+      <c r="P33" s="36">
         <f>IF(A33="","",N33-O33)</f>
         <v/>
       </c>
       <c r="Q33" s="4" t="n"/>
-      <c r="R33" s="14">
+      <c r="R33" s="36">
         <f>IF(A33="","",N(H33)+N(I33)+N(J33)+N(K33)+N(L33)+N33)</f>
         <v/>
       </c>
@@ -2742,36 +2757,36 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="n"/>
+      <c r="A34" s="35" t="n"/>
       <c r="B34" s="4" t="n"/>
       <c r="C34" s="4" t="n"/>
       <c r="D34" s="4" t="n"/>
       <c r="E34" s="4" t="n"/>
       <c r="F34" s="4" t="n"/>
       <c r="G34" s="4" t="n"/>
-      <c r="H34" s="14">
+      <c r="H34" s="36">
         <f>IF(G34="","",G34*$C$7)</f>
         <v/>
       </c>
-      <c r="I34" s="15" t="n"/>
-      <c r="J34" s="15" t="n"/>
-      <c r="K34" s="15" t="n"/>
-      <c r="L34" s="15" t="n"/>
+      <c r="I34" s="37" t="n"/>
+      <c r="J34" s="37" t="n"/>
+      <c r="K34" s="37" t="n"/>
+      <c r="L34" s="37" t="n"/>
       <c r="M34" s="4" t="n"/>
-      <c r="N34" s="14">
+      <c r="N34" s="36">
         <f>IF(A34="","",IF(COUNTIF($A$15:A34,A34)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O34" s="14">
+      <c r="O34" s="36">
         <f>IF(A34="","",MIN(N34,IF(AND(SUMIF($A$15:$A$39,A34,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A34,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A34,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A34,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P34" s="14">
+      <c r="P34" s="36">
         <f>IF(A34="","",N34-O34)</f>
         <v/>
       </c>
       <c r="Q34" s="4" t="n"/>
-      <c r="R34" s="14">
+      <c r="R34" s="36">
         <f>IF(A34="","",N(H34)+N(I34)+N(J34)+N(K34)+N(L34)+N34)</f>
         <v/>
       </c>
@@ -2781,36 +2796,36 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="n"/>
+      <c r="A35" s="35" t="n"/>
       <c r="B35" s="4" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="4" t="n"/>
       <c r="E35" s="4" t="n"/>
       <c r="F35" s="4" t="n"/>
       <c r="G35" s="4" t="n"/>
-      <c r="H35" s="14">
+      <c r="H35" s="36">
         <f>IF(G35="","",G35*$C$7)</f>
         <v/>
       </c>
-      <c r="I35" s="15" t="n"/>
-      <c r="J35" s="15" t="n"/>
-      <c r="K35" s="15" t="n"/>
-      <c r="L35" s="15" t="n"/>
+      <c r="I35" s="37" t="n"/>
+      <c r="J35" s="37" t="n"/>
+      <c r="K35" s="37" t="n"/>
+      <c r="L35" s="37" t="n"/>
       <c r="M35" s="4" t="n"/>
-      <c r="N35" s="14">
+      <c r="N35" s="36">
         <f>IF(A35="","",IF(COUNTIF($A$15:A35,A35)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O35" s="14">
+      <c r="O35" s="36">
         <f>IF(A35="","",MIN(N35,IF(AND(SUMIF($A$15:$A$39,A35,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A35,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A35,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A35,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P35" s="14">
+      <c r="P35" s="36">
         <f>IF(A35="","",N35-O35)</f>
         <v/>
       </c>
       <c r="Q35" s="4" t="n"/>
-      <c r="R35" s="14">
+      <c r="R35" s="36">
         <f>IF(A35="","",N(H35)+N(I35)+N(J35)+N(K35)+N(L35)+N35)</f>
         <v/>
       </c>
@@ -2820,36 +2835,36 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="13" t="n"/>
+      <c r="A36" s="35" t="n"/>
       <c r="B36" s="4" t="n"/>
       <c r="C36" s="4" t="n"/>
       <c r="D36" s="4" t="n"/>
       <c r="E36" s="4" t="n"/>
       <c r="F36" s="4" t="n"/>
       <c r="G36" s="4" t="n"/>
-      <c r="H36" s="14">
+      <c r="H36" s="36">
         <f>IF(G36="","",G36*$C$7)</f>
         <v/>
       </c>
-      <c r="I36" s="15" t="n"/>
-      <c r="J36" s="15" t="n"/>
-      <c r="K36" s="15" t="n"/>
-      <c r="L36" s="15" t="n"/>
+      <c r="I36" s="37" t="n"/>
+      <c r="J36" s="37" t="n"/>
+      <c r="K36" s="37" t="n"/>
+      <c r="L36" s="37" t="n"/>
       <c r="M36" s="4" t="n"/>
-      <c r="N36" s="14">
+      <c r="N36" s="36">
         <f>IF(A36="","",IF(COUNTIF($A$15:A36,A36)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O36" s="14">
+      <c r="O36" s="36">
         <f>IF(A36="","",MIN(N36,IF(AND(SUMIF($A$15:$A$39,A36,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A36,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A36,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A36,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P36" s="14">
+      <c r="P36" s="36">
         <f>IF(A36="","",N36-O36)</f>
         <v/>
       </c>
       <c r="Q36" s="4" t="n"/>
-      <c r="R36" s="14">
+      <c r="R36" s="36">
         <f>IF(A36="","",N(H36)+N(I36)+N(J36)+N(K36)+N(L36)+N36)</f>
         <v/>
       </c>
@@ -2859,36 +2874,36 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="n"/>
+      <c r="A37" s="35" t="n"/>
       <c r="B37" s="4" t="n"/>
       <c r="C37" s="4" t="n"/>
       <c r="D37" s="4" t="n"/>
       <c r="E37" s="4" t="n"/>
       <c r="F37" s="4" t="n"/>
       <c r="G37" s="4" t="n"/>
-      <c r="H37" s="14">
+      <c r="H37" s="36">
         <f>IF(G37="","",G37*$C$7)</f>
         <v/>
       </c>
-      <c r="I37" s="15" t="n"/>
-      <c r="J37" s="15" t="n"/>
-      <c r="K37" s="15" t="n"/>
-      <c r="L37" s="15" t="n"/>
+      <c r="I37" s="37" t="n"/>
+      <c r="J37" s="37" t="n"/>
+      <c r="K37" s="37" t="n"/>
+      <c r="L37" s="37" t="n"/>
       <c r="M37" s="4" t="n"/>
-      <c r="N37" s="14">
+      <c r="N37" s="36">
         <f>IF(A37="","",IF(COUNTIF($A$15:A37,A37)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O37" s="14">
+      <c r="O37" s="36">
         <f>IF(A37="","",MIN(N37,IF(AND(SUMIF($A$15:$A$39,A37,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A37,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A37,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A37,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P37" s="14">
+      <c r="P37" s="36">
         <f>IF(A37="","",N37-O37)</f>
         <v/>
       </c>
       <c r="Q37" s="4" t="n"/>
-      <c r="R37" s="14">
+      <c r="R37" s="36">
         <f>IF(A37="","",N(H37)+N(I37)+N(J37)+N(K37)+N(L37)+N37)</f>
         <v/>
       </c>
@@ -2898,36 +2913,36 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="n"/>
+      <c r="A38" s="35" t="n"/>
       <c r="B38" s="4" t="n"/>
       <c r="C38" s="4" t="n"/>
       <c r="D38" s="4" t="n"/>
       <c r="E38" s="4" t="n"/>
       <c r="F38" s="4" t="n"/>
       <c r="G38" s="4" t="n"/>
-      <c r="H38" s="14">
+      <c r="H38" s="36">
         <f>IF(G38="","",G38*$C$7)</f>
         <v/>
       </c>
-      <c r="I38" s="15" t="n"/>
-      <c r="J38" s="15" t="n"/>
-      <c r="K38" s="15" t="n"/>
-      <c r="L38" s="15" t="n"/>
+      <c r="I38" s="37" t="n"/>
+      <c r="J38" s="37" t="n"/>
+      <c r="K38" s="37" t="n"/>
+      <c r="L38" s="37" t="n"/>
       <c r="M38" s="4" t="n"/>
-      <c r="N38" s="14">
+      <c r="N38" s="36">
         <f>IF(A38="","",IF(COUNTIF($A$15:A38,A38)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O38" s="14">
+      <c r="O38" s="36">
         <f>IF(A38="","",MIN(N38,IF(AND(SUMIF($A$15:$A$39,A38,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A38,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A38,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A38,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P38" s="14">
+      <c r="P38" s="36">
         <f>IF(A38="","",N38-O38)</f>
         <v/>
       </c>
       <c r="Q38" s="4" t="n"/>
-      <c r="R38" s="14">
+      <c r="R38" s="36">
         <f>IF(A38="","",N(H38)+N(I38)+N(J38)+N(K38)+N(L38)+N38)</f>
         <v/>
       </c>
@@ -2937,36 +2952,36 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="13" t="n"/>
+      <c r="A39" s="35" t="n"/>
       <c r="B39" s="4" t="n"/>
       <c r="C39" s="4" t="n"/>
       <c r="D39" s="4" t="n"/>
       <c r="E39" s="4" t="n"/>
       <c r="F39" s="4" t="n"/>
       <c r="G39" s="4" t="n"/>
-      <c r="H39" s="14">
+      <c r="H39" s="36">
         <f>IF(G39="","",G39*$C$7)</f>
         <v/>
       </c>
-      <c r="I39" s="15" t="n"/>
-      <c r="J39" s="15" t="n"/>
-      <c r="K39" s="15" t="n"/>
-      <c r="L39" s="15" t="n"/>
+      <c r="I39" s="37" t="n"/>
+      <c r="J39" s="37" t="n"/>
+      <c r="K39" s="37" t="n"/>
+      <c r="L39" s="37" t="n"/>
       <c r="M39" s="4" t="n"/>
-      <c r="N39" s="14">
+      <c r="N39" s="36">
         <f>IF(A39="","",IF(COUNTIF($A$15:A39,A39)=1,$C$8,0))</f>
         <v/>
       </c>
-      <c r="O39" s="14">
+      <c r="O39" s="36">
         <f>IF(A39="","",MIN(N39,IF(AND(SUMIF($A$15:$A$39,A39,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A39,$L$15:$L$39)&gt;0),$C$11,IF(OR(SUMIF($A$15:$A$39,A39,$K$15:$K$39)&gt;0,SUMIF($A$15:$A$39,A39,$L$15:$L$39)&gt;0),$C$10,$C$9))))</f>
         <v/>
       </c>
-      <c r="P39" s="14">
+      <c r="P39" s="36">
         <f>IF(A39="","",N39-O39)</f>
         <v/>
       </c>
       <c r="Q39" s="4" t="n"/>
-      <c r="R39" s="14">
+      <c r="R39" s="36">
         <f>IF(A39="","",N(H39)+N(I39)+N(J39)+N(K39)+N(L39)+N39)</f>
         <v/>
       </c>
@@ -2975,7 +2990,6 @@
         <v/>
       </c>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="F41" s="3" t="inlineStr">
         <is>
@@ -2986,39 +3000,39 @@
         <f>SUM(G15:G39)</f>
         <v/>
       </c>
-      <c r="H41" s="18">
+      <c r="H41" s="38">
         <f>SUM(H15:H39)</f>
         <v/>
       </c>
-      <c r="I41" s="18">
+      <c r="I41" s="38">
         <f>SUM(I15:I39)</f>
         <v/>
       </c>
-      <c r="J41" s="18">
+      <c r="J41" s="38">
         <f>SUM(J15:J39)</f>
         <v/>
       </c>
-      <c r="K41" s="18">
+      <c r="K41" s="38">
         <f>SUM(K15:K39)</f>
         <v/>
       </c>
-      <c r="L41" s="18">
+      <c r="L41" s="38">
         <f>SUM(L15:L39)</f>
         <v/>
       </c>
-      <c r="N41" s="18">
+      <c r="N41" s="38">
         <f>SUM(N15:N39)</f>
         <v/>
       </c>
-      <c r="O41" s="18">
+      <c r="O41" s="38">
         <f>SUM(O15:O39)</f>
         <v/>
       </c>
-      <c r="P41" s="18">
+      <c r="P41" s="38">
         <f>SUM(P15:P39)</f>
         <v/>
       </c>
-      <c r="R41" s="18">
+      <c r="R41" s="38">
         <f>SUM(R15:R39)</f>
         <v/>
       </c>
@@ -3029,7 +3043,7 @@
           <t>DA PAGARE (solo righe OK)</t>
         </is>
       </c>
-      <c r="R42" s="19">
+      <c r="R42" s="39">
         <f>SUMIFS(R15:R39,S15:S39,"OK")</f>
         <v/>
       </c>
@@ -3040,7 +3054,7 @@
           <t>di cui da tassare in cedolino (indennità oltre soglia, righe OK)</t>
         </is>
       </c>
-      <c r="R43" s="27">
+      <c r="R43" s="43">
         <f>SUMIFS(P15:P39,S15:S39,"OK")</f>
         <v/>
       </c>
@@ -3056,8 +3070,6 @@
         <v/>
       </c>
     </row>
-    <row r="45"/>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
@@ -3070,7 +3082,6 @@
       <c r="F47" s="21" t="n"/>
       <c r="G47" s="21" t="n"/>
     </row>
-    <row r="48"/>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
@@ -3083,7 +3094,6 @@
       <c r="F49" s="21" t="n"/>
       <c r="G49" s="21" t="n"/>
     </row>
-    <row r="50"/>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
@@ -3096,7 +3106,6 @@
       <c r="F51" s="21" t="n"/>
       <c r="G51" s="21" t="n"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
@@ -3255,7 +3264,7 @@
     <row r="18">
       <c r="A18" s="29" t="inlineStr">
         <is>
-          <t>- Tragitto casa-lavoro (Verona - Villafranca nei giorni in ufficio): non è trasferta, è reddito.</t>
+          <t>- Tragitto casa-lavoro (Verona - Villafranca nei giorni in ufficio): non è una trasferta.</t>
         </is>
       </c>
     </row>
@@ -3269,7 +3278,7 @@
     <row r="20">
       <c r="A20" s="29" t="inlineStr">
         <is>
-          <t>- Contributi INPS personali, spese per marchi, spese personali di qualunque tipo.</t>
+          <t>- Qualsiasi spesa personale o non legata a una trasferta. Se una spesa riguarda Overall, la paga Overall con fattura intestata alla società.</t>
         </is>
       </c>
     </row>
@@ -3283,7 +3292,7 @@
     <row r="22">
       <c r="A22" s="29" t="inlineStr">
         <is>
-          <t>- Km stimati o «ricostruiti» per arrivare a una cifra; importi tondi o identici ogni mese.</t>
+          <t>- Importi senza documento: ogni cifra viene dal percorso stampato o da una ricevuta.</t>
         </is>
       </c>
     </row>

</xml_diff>